<commit_message>
fix: F1-F7 code review fixes — lock file, raw date, unified parser, pincode race, section numbering, defaults caching, unused import
</commit_message>
<xml_diff>
--- a/OIC DOCS/dummy.xlsx
+++ b/OIC DOCS/dummy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jadav\Coding\Automation\UIIC\uiic_automation\OIC DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5326ED0-966D-43F8-9EA0-DA4F750134E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F7E54A8-0A55-492C-B48E-CD41D68BDD3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{0249C969-0BD7-4CC8-B38D-D9EE02361E7A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="236">
   <si>
     <t>Type of Body</t>
   </si>
@@ -331,9 +331,6 @@
     <t>Type of Licence</t>
   </si>
   <si>
-    <t>LMV-MCWG</t>
-  </si>
-  <si>
     <t>initial loss assessment</t>
   </si>
   <si>
@@ -697,9 +694,6 @@
     <t>AGRA</t>
   </si>
   <si>
-    <t>Panchkula, Haryana</t>
-  </si>
-  <si>
     <t xml:space="preserve">pin code </t>
   </si>
   <si>
@@ -722,6 +716,36 @@
   </si>
   <si>
     <t>CBZL12533</t>
+  </si>
+  <si>
+    <t>RTO NAME</t>
+  </si>
+  <si>
+    <t>gaya</t>
+  </si>
+  <si>
+    <t>workshop date</t>
+  </si>
+  <si>
+    <t>HPV</t>
+  </si>
+  <si>
+    <t>registered_owner_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">workshop estimate date </t>
+  </si>
+  <si>
+    <t xml:space="preserve">expiry date </t>
+  </si>
+  <si>
+    <t>license_number</t>
+  </si>
+  <si>
+    <t>SLA/200019</t>
+  </si>
+  <si>
+    <t>assam, bajali</t>
   </si>
 </sst>
 </file>
@@ -729,11 +753,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
-    <numFmt numFmtId="165" formatCode="[$-409]mmmmm\-yy;@"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="m/d/yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="[$-409]mmmmm\-yy;@"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -788,6 +812,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFD7BA7D"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1075,7 +1105,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="140">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1089,10 +1119,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1153,7 +1183,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1293,45 +1323,47 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="justify"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1360,16 +1392,16 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>4</xdr:col>
-          <xdr:colOff>1524</xdr:colOff>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>597408</xdr:colOff>
           <xdr:row>194</xdr:row>
-          <xdr:rowOff>158496</xdr:rowOff>
+          <xdr:rowOff>173736</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>291084</xdr:colOff>
+          <xdr:colOff>179832</xdr:colOff>
           <xdr:row>196</xdr:row>
-          <xdr:rowOff>67056</xdr:rowOff>
+          <xdr:rowOff>82296</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1710,12 +1742,14 @@
   <dimension ref="A2:AE294"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="8.77734375" style="1"/>
+    <col min="1" max="3" width="8.77734375" style="1"/>
+    <col min="4" max="4" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="8.77734375" style="1"/>
     <col min="7" max="7" width="26.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="23.77734375" style="1" customWidth="1"/>
-    <col min="9" max="13" width="8.77734375" style="1"/>
+    <col min="9" max="9" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="13" width="8.77734375" style="1"/>
     <col min="14" max="14" width="25.109375" style="1" customWidth="1"/>
     <col min="15" max="15" width="32" style="1" customWidth="1"/>
     <col min="16" max="16384" width="8.77734375" style="1"/>
@@ -2077,18 +2111,18 @@
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
-      <c r="B12" s="129" t="s">
+      <c r="B12" s="130" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="130"/>
-      <c r="D12" s="130"/>
-      <c r="E12" s="130"/>
-      <c r="F12" s="130"/>
-      <c r="G12" s="130"/>
-      <c r="H12" s="130"/>
-      <c r="I12" s="130"/>
-      <c r="J12" s="130"/>
-      <c r="K12" s="130"/>
+      <c r="C12" s="131"/>
+      <c r="D12" s="131"/>
+      <c r="E12" s="131"/>
+      <c r="F12" s="131"/>
+      <c r="G12" s="131"/>
+      <c r="H12" s="131"/>
+      <c r="I12" s="131"/>
+      <c r="J12" s="131"/>
+      <c r="K12" s="131"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
@@ -2623,7 +2657,7 @@
         <v>19</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="4"/>
@@ -2664,7 +2698,7 @@
         <v>19</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
@@ -2739,14 +2773,14 @@
       <c r="D29" s="19"/>
       <c r="E29" s="20"/>
       <c r="F29" s="21"/>
-      <c r="G29" s="134" t="s">
+      <c r="G29" s="126" t="s">
         <v>41</v>
       </c>
-      <c r="H29" s="133"/>
-      <c r="I29" s="136" t="s">
+      <c r="H29" s="127"/>
+      <c r="I29" s="132" t="s">
         <v>42</v>
       </c>
-      <c r="J29" s="133"/>
+      <c r="J29" s="127"/>
       <c r="K29" s="22" t="s">
         <v>43</v>
       </c>
@@ -2784,15 +2818,15 @@
       <c r="F30" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="G30" s="137" t="s">
-        <v>226</v>
-      </c>
-      <c r="H30" s="126"/>
-      <c r="I30" s="136" t="str">
+      <c r="G30" s="133" t="s">
+        <v>224</v>
+      </c>
+      <c r="H30" s="134"/>
+      <c r="I30" s="132" t="str">
         <f>G30</f>
         <v>MEXC19606KT080595</v>
       </c>
-      <c r="J30" s="133"/>
+      <c r="J30" s="127"/>
       <c r="K30" s="22" t="str">
         <f>G30</f>
         <v>MEXC19606KT080595</v>
@@ -2831,15 +2865,15 @@
       <c r="F31" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="G31" s="134" t="s">
-        <v>227</v>
-      </c>
-      <c r="H31" s="133"/>
-      <c r="I31" s="135" t="str">
+      <c r="G31" s="126" t="s">
+        <v>225</v>
+      </c>
+      <c r="H31" s="127"/>
+      <c r="I31" s="128" t="str">
         <f>G31</f>
         <v>CBZL12533</v>
       </c>
-      <c r="J31" s="128"/>
+      <c r="J31" s="129"/>
       <c r="K31" s="27" t="str">
         <f>G31</f>
         <v>CBZL12533</v>
@@ -2879,7 +2913,7 @@
         <v>19</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -3283,8 +3317,12 @@
       <c r="G42" s="2">
         <v>54</v>
       </c>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
+      <c r="H42" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>227</v>
+      </c>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
@@ -3533,8 +3571,12 @@
       <c r="G48" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="H48" s="2"/>
-      <c r="I48" s="2"/>
+      <c r="H48" s="139" t="s">
+        <v>230</v>
+      </c>
+      <c r="I48" s="125" t="s">
+        <v>81</v>
+      </c>
       <c r="J48" s="8" t="s">
         <v>82</v>
       </c>
@@ -3615,7 +3657,7 @@
         <v>19</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
@@ -3826,7 +3868,7 @@
         <v>19</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>97</v>
+        <v>229</v>
       </c>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
@@ -3868,7 +3910,7 @@
       <c r="L56" s="2"/>
       <c r="M56" s="2"/>
       <c r="N56" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O56" s="2">
         <v>50000</v>
@@ -3896,7 +3938,7 @@
         <v>4</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="32"/>
@@ -3909,10 +3951,10 @@
       <c r="L57" s="2"/>
       <c r="M57" s="2"/>
       <c r="N57" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O57" s="122" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P57" s="2"/>
       <c r="Q57" s="2"/>
@@ -3937,7 +3979,7 @@
         <v>17</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="13"/>
@@ -3978,7 +4020,7 @@
         <v>23</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="13"/>
@@ -3986,7 +4028,7 @@
         <v>19</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
@@ -4028,7 +4070,7 @@
       <c r="L60" s="2"/>
       <c r="M60" s="2"/>
       <c r="N60" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="O60" s="123">
         <v>0.42708333333333331</v>
@@ -4056,7 +4098,7 @@
         <v>5</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="32"/>
@@ -4069,7 +4111,7 @@
       <c r="L61" s="2"/>
       <c r="M61" s="2"/>
       <c r="N61" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="O61" s="2">
         <v>987</v>
@@ -4095,7 +4137,7 @@
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="13"/>
@@ -4112,7 +4154,7 @@
       <c r="L62" s="2"/>
       <c r="M62" s="2"/>
       <c r="N62" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="O62" s="2">
         <v>781371</v>
@@ -4138,7 +4180,7 @@
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="13"/>
@@ -4146,10 +4188,10 @@
         <v>19</v>
       </c>
       <c r="G63" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H63" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="H63" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
@@ -4157,10 +4199,10 @@
       <c r="L63" s="2"/>
       <c r="M63" s="2"/>
       <c r="N63" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="O63" s="122" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="P63" s="2"/>
       <c r="Q63" s="2"/>
@@ -4183,7 +4225,7 @@
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="32"/>
@@ -4191,7 +4233,7 @@
         <v>19</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
@@ -4222,7 +4264,7 @@
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="13"/>
@@ -4230,7 +4272,7 @@
         <v>19</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
@@ -4329,7 +4371,7 @@
         <v>6</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D68" s="2"/>
       <c r="E68" s="4"/>
@@ -4364,7 +4406,7 @@
       <c r="A69" s="2"/>
       <c r="B69" s="14"/>
       <c r="C69" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D69" s="2"/>
       <c r="E69" s="4"/>
@@ -4372,10 +4414,14 @@
         <v>19</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H69" s="2"/>
-      <c r="I69" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I69" s="124">
+        <v>46149</v>
+      </c>
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
       <c r="L69" s="2"/>
@@ -4411,7 +4457,7 @@
         <v>19</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
@@ -4442,7 +4488,7 @@
       <c r="A71" s="2"/>
       <c r="B71" s="14"/>
       <c r="C71" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D71" s="2"/>
       <c r="E71" s="4"/>
@@ -4450,7 +4496,7 @@
         <v>19</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
@@ -4480,8 +4526,12 @@
     <row r="72" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
+      <c r="C72" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D72" s="124">
+        <v>46152</v>
+      </c>
       <c r="E72" s="2"/>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
@@ -4516,7 +4566,7 @@
         <v>7</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D73" s="2"/>
       <c r="E73" s="13"/>
@@ -4524,7 +4574,7 @@
         <v>19</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
@@ -4590,7 +4640,7 @@
         <v>8</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D75" s="2"/>
       <c r="E75" s="13"/>
@@ -4598,7 +4648,7 @@
         <v>19</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
@@ -4664,7 +4714,7 @@
         <v>9</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D77" s="2"/>
       <c r="E77" s="32"/>
@@ -4699,7 +4749,7 @@
       <c r="A78" s="2"/>
       <c r="B78" s="14"/>
       <c r="C78" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D78" s="2"/>
       <c r="E78" s="32"/>
@@ -4733,17 +4783,17 @@
     <row r="79" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A79" s="2"/>
       <c r="B79" s="14"/>
-      <c r="C79" s="129" t="s">
+      <c r="C79" s="130" t="s">
         <v>20</v>
       </c>
-      <c r="D79" s="130"/>
-      <c r="E79" s="130"/>
-      <c r="F79" s="130"/>
-      <c r="G79" s="130"/>
-      <c r="H79" s="130"/>
-      <c r="I79" s="130"/>
-      <c r="J79" s="130"/>
-      <c r="K79" s="130"/>
+      <c r="D79" s="131"/>
+      <c r="E79" s="131"/>
+      <c r="F79" s="131"/>
+      <c r="G79" s="131"/>
+      <c r="H79" s="131"/>
+      <c r="I79" s="131"/>
+      <c r="J79" s="131"/>
+      <c r="K79" s="131"/>
       <c r="L79" s="2"/>
       <c r="M79" s="2"/>
       <c r="N79" s="2"/>
@@ -4773,8 +4823,12 @@
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
-      <c r="H80" s="2"/>
-      <c r="I80" s="2"/>
+      <c r="H80" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I80" s="124">
+        <v>46169</v>
+      </c>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
       <c r="L80" s="2"/>
@@ -4804,14 +4858,18 @@
         <v>10</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
-      <c r="H81" s="2"/>
-      <c r="I81" s="2"/>
+      <c r="H81" s="125" t="s">
+        <v>233</v>
+      </c>
+      <c r="I81" s="125" t="s">
+        <v>234</v>
+      </c>
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
       <c r="L81" s="2"/>
@@ -4838,17 +4896,17 @@
     <row r="82" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A82" s="2"/>
       <c r="B82" s="14"/>
-      <c r="C82" s="129" t="s">
-        <v>124</v>
-      </c>
-      <c r="D82" s="130"/>
-      <c r="E82" s="130"/>
-      <c r="F82" s="130"/>
-      <c r="G82" s="130"/>
-      <c r="H82" s="130"/>
-      <c r="I82" s="130"/>
-      <c r="J82" s="130"/>
-      <c r="K82" s="130"/>
+      <c r="C82" s="130" t="s">
+        <v>123</v>
+      </c>
+      <c r="D82" s="131"/>
+      <c r="E82" s="131"/>
+      <c r="F82" s="131"/>
+      <c r="G82" s="131"/>
+      <c r="H82" s="131"/>
+      <c r="I82" s="131"/>
+      <c r="J82" s="131"/>
+      <c r="K82" s="131"/>
       <c r="L82" s="2"/>
       <c r="M82" s="2"/>
       <c r="N82" s="2"/>
@@ -4909,7 +4967,7 @@
         <v>11</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
@@ -4944,7 +5002,7 @@
       <c r="A85" s="2"/>
       <c r="B85" s="14"/>
       <c r="C85" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D85" s="2"/>
       <c r="E85" s="2"/>
@@ -5014,7 +5072,7 @@
         <v>12</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
@@ -5088,7 +5146,7 @@
         <v>2</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
@@ -5125,7 +5183,7 @@
         <v>3</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="2"/>
@@ -5162,7 +5220,7 @@
         <v>4</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D91" s="2"/>
       <c r="E91" s="2"/>
@@ -5232,7 +5290,7 @@
         <v>13</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D93" s="2"/>
       <c r="E93" s="2"/>
@@ -5301,7 +5359,7 @@
       <c r="B95" s="18"/>
       <c r="C95" s="19"/>
       <c r="D95" s="19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E95" s="19"/>
       <c r="F95" s="35"/>
@@ -5336,7 +5394,7 @@
     <row r="96" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
@@ -5346,7 +5404,7 @@
         <v>-119.88888888888889</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
@@ -5379,7 +5437,7 @@
     <row r="97" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
       <c r="B97" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C97" s="19"/>
       <c r="D97" s="19"/>
@@ -5388,7 +5446,7 @@
         <v>18</v>
       </c>
       <c r="G97" s="19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H97" s="19"/>
       <c r="I97" s="19"/>
@@ -5458,13 +5516,13 @@
       <c r="E99" s="5"/>
       <c r="F99" s="5"/>
       <c r="G99" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H99" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I99" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J99" s="2"/>
       <c r="K99" s="2"/>
@@ -5492,30 +5550,30 @@
     <row r="100" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C100" s="30" t="s">
         <v>138</v>
-      </c>
-      <c r="C100" s="30" t="s">
-        <v>139</v>
       </c>
       <c r="D100" s="5"/>
       <c r="E100" s="31"/>
       <c r="F100" s="42" t="s">
+        <v>139</v>
+      </c>
+      <c r="G100" s="42" t="s">
         <v>140</v>
       </c>
-      <c r="G100" s="42" t="s">
+      <c r="H100" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="H100" s="42" t="s">
+      <c r="I100" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="I100" s="43" t="s">
+      <c r="J100" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="J100" s="8" t="s">
+      <c r="K100" s="44" t="s">
         <v>144</v>
-      </c>
-      <c r="K100" s="44" t="s">
-        <v>145</v>
       </c>
       <c r="L100" s="2"/>
       <c r="M100" s="2"/>
@@ -5544,7 +5602,7 @@
         <v>1</v>
       </c>
       <c r="C101" s="45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D101" s="2"/>
       <c r="E101" s="38"/>
@@ -5587,7 +5645,7 @@
         <v>2</v>
       </c>
       <c r="C102" s="47" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D102" s="2"/>
       <c r="E102" s="38"/>
@@ -5630,7 +5688,7 @@
         <v>3</v>
       </c>
       <c r="C103" s="47" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D103" s="2"/>
       <c r="E103" s="38"/>
@@ -5638,7 +5696,7 @@
         <v>8570</v>
       </c>
       <c r="G103" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H103" s="46">
         <v>500</v>
@@ -5673,7 +5731,7 @@
         <v>4</v>
       </c>
       <c r="C104" s="47" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D104" s="2"/>
       <c r="E104" s="38"/>
@@ -5681,7 +5739,7 @@
         <v>8861</v>
       </c>
       <c r="G104" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H104" s="46">
         <v>5</v>
@@ -5716,7 +5774,7 @@
         <v>5</v>
       </c>
       <c r="C105" s="47" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D105" s="2"/>
       <c r="E105" s="38"/>
@@ -5724,7 +5782,7 @@
         <v>9110</v>
       </c>
       <c r="G105" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H105" s="46">
         <v>5</v>
@@ -5759,7 +5817,7 @@
         <v>6</v>
       </c>
       <c r="C106" s="47" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D106" s="2"/>
       <c r="E106" s="38"/>
@@ -5767,7 +5825,7 @@
         <v>3030</v>
       </c>
       <c r="G106" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H106" s="46">
         <v>4</v>
@@ -5802,7 +5860,7 @@
         <v>7</v>
       </c>
       <c r="C107" s="47" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D107" s="2"/>
       <c r="E107" s="38"/>
@@ -5810,7 +5868,7 @@
         <v>1560</v>
       </c>
       <c r="G107" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H107" s="46"/>
       <c r="I107" s="46">
@@ -5845,7 +5903,7 @@
         <v>8</v>
       </c>
       <c r="C108" s="47" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D108" s="2"/>
       <c r="E108" s="38"/>
@@ -5853,7 +5911,7 @@
         <v>8570</v>
       </c>
       <c r="G108" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H108" s="46">
         <v>4</v>
@@ -5888,7 +5946,7 @@
         <v>9</v>
       </c>
       <c r="C109" s="47" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D109" s="2"/>
       <c r="E109" s="38"/>
@@ -5896,7 +5954,7 @@
         <v>9110</v>
       </c>
       <c r="G109" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H109" s="46">
         <v>4</v>
@@ -5931,7 +5989,7 @@
         <v>10</v>
       </c>
       <c r="C110" s="47" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D110" s="2"/>
       <c r="E110" s="38"/>
@@ -5939,7 +5997,7 @@
         <v>8861</v>
       </c>
       <c r="G110" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H110" s="46"/>
       <c r="I110" s="46">
@@ -5974,7 +6032,7 @@
         <v>11</v>
       </c>
       <c r="C111" s="47" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D111" s="2"/>
       <c r="E111" s="38"/>
@@ -5982,7 +6040,7 @@
         <v>2270</v>
       </c>
       <c r="G111" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H111" s="46"/>
       <c r="I111" s="46">
@@ -6017,7 +6075,7 @@
         <v>12</v>
       </c>
       <c r="C112" s="47" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D112" s="2"/>
       <c r="E112" s="38"/>
@@ -6025,7 +6083,7 @@
         <v>2270</v>
       </c>
       <c r="G112" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H112" s="46">
         <v>5</v>
@@ -6060,7 +6118,7 @@
         <v>13</v>
       </c>
       <c r="C113" s="47" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D113" s="2"/>
       <c r="E113" s="38"/>
@@ -6068,7 +6126,7 @@
         <v>302</v>
       </c>
       <c r="G113" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H113" s="46">
         <v>4</v>
@@ -6103,7 +6161,7 @@
         <v>14</v>
       </c>
       <c r="C114" s="47" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D114" s="2"/>
       <c r="E114" s="38"/>
@@ -6111,7 +6169,7 @@
         <v>3560</v>
       </c>
       <c r="G114" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H114" s="46"/>
       <c r="I114" s="46">
@@ -6146,7 +6204,7 @@
         <v>15</v>
       </c>
       <c r="C115" s="47" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D115" s="2"/>
       <c r="E115" s="38"/>
@@ -6154,7 +6212,7 @@
         <v>70000</v>
       </c>
       <c r="G115" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H115" s="46">
         <v>4</v>
@@ -6189,7 +6247,7 @@
         <v>16</v>
       </c>
       <c r="C116" s="47" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D116" s="2"/>
       <c r="E116" s="38"/>
@@ -6234,7 +6292,7 @@
         <v>17</v>
       </c>
       <c r="C117" s="47" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D117" s="2"/>
       <c r="E117" s="38"/>
@@ -6872,7 +6930,7 @@
     <row r="136" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A136" s="2"/>
       <c r="B136" s="23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C136" s="2"/>
       <c r="D136" s="2"/>
@@ -6925,7 +6983,7 @@
         <v>18</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D137" s="5"/>
       <c r="E137" s="31"/>
@@ -6971,7 +7029,7 @@
     <row r="138" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A138" s="2"/>
       <c r="B138" s="23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" s="2"/>
@@ -7018,7 +7076,7 @@
     <row r="139" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A139" s="2"/>
       <c r="B139" s="61" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C139" s="2"/>
       <c r="D139" s="2"/>
@@ -7057,7 +7115,7 @@
         <v>0</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D140" s="5"/>
       <c r="E140" s="31"/>
@@ -7099,7 +7157,7 @@
     <row r="141" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A141" s="2"/>
       <c r="B141" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C141" s="19"/>
       <c r="D141" s="19"/>
@@ -7146,7 +7204,7 @@
     <row r="142" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A142" s="2"/>
       <c r="B142" s="30" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C142" s="5"/>
       <c r="D142" s="19"/>
@@ -7220,7 +7278,7 @@
     <row r="144" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A144" s="2"/>
       <c r="B144" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C144" s="2"/>
       <c r="D144" s="2"/>
@@ -7522,7 +7580,7 @@
     <row r="153" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A153" s="2"/>
       <c r="B153" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C153" s="2"/>
       <c r="D153" s="2"/>
@@ -7590,7 +7648,7 @@
     <row r="155" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A155" s="2"/>
       <c r="B155" s="70" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C155" s="19"/>
       <c r="D155" s="19"/>
@@ -7625,24 +7683,24 @@
     <row r="156" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A156" s="2"/>
       <c r="B156" s="73" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C156" s="74" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D156" s="19"/>
       <c r="E156" s="36"/>
       <c r="F156" s="75" t="s">
+        <v>173</v>
+      </c>
+      <c r="G156" s="76" t="s">
         <v>174</v>
       </c>
-      <c r="G156" s="76" t="s">
+      <c r="H156" s="77" t="s">
         <v>175</v>
       </c>
-      <c r="H156" s="77" t="s">
+      <c r="I156" s="78" t="s">
         <v>176</v>
-      </c>
-      <c r="I156" s="78" t="s">
-        <v>177</v>
       </c>
       <c r="J156" s="2"/>
       <c r="K156" s="2"/>
@@ -7673,7 +7731,7 @@
         <v>1</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D157" s="2"/>
       <c r="E157" s="2"/>
@@ -7712,7 +7770,7 @@
         <v>2</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D158" s="2"/>
       <c r="E158" s="2"/>
@@ -7751,7 +7809,7 @@
         <v>3</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D159" s="2"/>
       <c r="E159" s="2"/>
@@ -7853,7 +7911,7 @@
     <row r="162" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A162" s="2"/>
       <c r="B162" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C162" s="41"/>
       <c r="D162" s="41"/>
@@ -7933,7 +7991,7 @@
     <row r="164" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A164" s="38"/>
       <c r="B164" s="70" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C164" s="19"/>
       <c r="D164" s="19"/>
@@ -7982,7 +8040,7 @@
       <c r="B165" s="30"/>
       <c r="C165" s="5"/>
       <c r="D165" s="49" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E165" s="5"/>
       <c r="F165" s="86"/>
@@ -8051,7 +8109,7 @@
     <row r="167" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A167" s="2"/>
       <c r="B167" s="70" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C167" s="19"/>
       <c r="D167" s="19"/>
@@ -8059,10 +8117,10 @@
       <c r="F167" s="92"/>
       <c r="G167" s="92"/>
       <c r="H167" s="93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I167" s="93" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J167" s="2"/>
       <c r="K167" s="2"/>
@@ -8133,7 +8191,7 @@
         <v>18</v>
       </c>
       <c r="C169" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D169" s="2"/>
       <c r="E169" s="2"/>
@@ -8173,7 +8231,7 @@
     <row r="170" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A170" s="2"/>
       <c r="B170" s="70" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C170" s="19"/>
       <c r="D170" s="19"/>
@@ -8247,7 +8305,7 @@
     <row r="172" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A172" s="2"/>
       <c r="B172" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C172" s="2"/>
       <c r="D172" s="2"/>
@@ -8318,16 +8376,16 @@
     <row r="174" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A174" s="2"/>
       <c r="B174" s="30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C174" s="5"/>
       <c r="D174" s="5"/>
       <c r="E174" s="31"/>
       <c r="F174" s="42" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G174" s="42" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H174" s="2"/>
       <c r="I174" s="2"/>
@@ -8357,7 +8415,7 @@
     <row r="175" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A175" s="2"/>
       <c r="B175" s="97" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C175" s="41"/>
       <c r="D175" s="41"/>
@@ -8398,7 +8456,7 @@
     <row r="176" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A176" s="2"/>
       <c r="B176" s="24" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C176" s="5"/>
       <c r="D176" s="5"/>
@@ -8439,7 +8497,7 @@
     <row r="177" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A177" s="2"/>
       <c r="B177" s="23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="2"/>
@@ -8480,7 +8538,7 @@
     <row r="178" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A178" s="2"/>
       <c r="B178" s="24" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C178" s="5"/>
       <c r="D178" s="5"/>
@@ -8518,7 +8576,7 @@
     <row r="179" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A179" s="2"/>
       <c r="B179" s="30" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C179" s="5"/>
       <c r="D179" s="19"/>
@@ -8592,7 +8650,7 @@
     <row r="181" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A181" s="2"/>
       <c r="B181" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C181" s="2"/>
       <c r="D181" s="2"/>
@@ -8629,7 +8687,7 @@
     <row r="182" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A182" s="2"/>
       <c r="B182" s="70" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C182" s="19"/>
       <c r="D182" s="19"/>
@@ -8699,18 +8757,18 @@
     </row>
     <row r="184" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A184" s="33"/>
-      <c r="B184" s="131" t="s">
-        <v>190</v>
-      </c>
-      <c r="C184" s="130"/>
-      <c r="D184" s="130"/>
-      <c r="E184" s="130"/>
-      <c r="F184" s="130"/>
-      <c r="G184" s="130"/>
-      <c r="H184" s="130"/>
-      <c r="I184" s="130"/>
-      <c r="J184" s="130"/>
-      <c r="K184" s="130"/>
+      <c r="B184" s="137" t="s">
+        <v>189</v>
+      </c>
+      <c r="C184" s="131"/>
+      <c r="D184" s="131"/>
+      <c r="E184" s="131"/>
+      <c r="F184" s="131"/>
+      <c r="G184" s="131"/>
+      <c r="H184" s="131"/>
+      <c r="I184" s="131"/>
+      <c r="J184" s="131"/>
+      <c r="K184" s="131"/>
       <c r="L184" s="2"/>
       <c r="M184" s="2"/>
       <c r="N184" s="2"/>
@@ -8768,7 +8826,7 @@
     <row r="186" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A186" s="2"/>
       <c r="B186" s="100" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="2"/>
@@ -8839,7 +8897,7 @@
         <v>1</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D188" s="2"/>
       <c r="E188" s="4" t="s">
@@ -8914,7 +8972,7 @@
         <v>2</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D190" s="2"/>
       <c r="E190" s="4" t="s">
@@ -8987,7 +9045,7 @@
       <c r="A192" s="2"/>
       <c r="B192" s="4"/>
       <c r="C192" s="97" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D192" s="41"/>
       <c r="E192" s="41"/>
@@ -8996,7 +9054,7 @@
       <c r="H192" s="2"/>
       <c r="I192" s="2"/>
       <c r="J192" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K192" s="2"/>
       <c r="L192" s="2"/>
@@ -9057,7 +9115,7 @@
       <c r="A194" s="2"/>
       <c r="B194" s="4"/>
       <c r="C194" s="102" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D194" s="5"/>
       <c r="E194" s="5"/>
@@ -9191,13 +9249,13 @@
       <c r="A198" s="2"/>
       <c r="B198" s="2"/>
       <c r="C198" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D198" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E198" s="121" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F198" s="120">
         <v>3.5010231260389999E+19</v>
@@ -9211,7 +9269,7 @@
       <c r="K198" s="2"/>
       <c r="L198" s="2"/>
       <c r="M198" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="N198" s="2"/>
       <c r="O198" s="2"/>
@@ -9279,27 +9337,27 @@
       <c r="K200" s="2"/>
       <c r="L200" s="2"/>
       <c r="M200" s="78" t="s">
+        <v>197</v>
+      </c>
+      <c r="N200" s="103" t="s">
         <v>198</v>
       </c>
-      <c r="N200" s="103" t="s">
+      <c r="O200" s="138" t="s">
         <v>199</v>
       </c>
-      <c r="O200" s="132" t="s">
+      <c r="P200" s="127"/>
+      <c r="Q200" s="138" t="s">
         <v>200</v>
       </c>
-      <c r="P200" s="133"/>
-      <c r="Q200" s="132" t="s">
+      <c r="R200" s="127"/>
+      <c r="S200" s="138" t="s">
         <v>201</v>
       </c>
-      <c r="R200" s="133"/>
-      <c r="S200" s="132" t="s">
+      <c r="T200" s="127"/>
+      <c r="U200" s="135" t="s">
         <v>202</v>
       </c>
-      <c r="T200" s="133"/>
-      <c r="U200" s="125" t="s">
-        <v>203</v>
-      </c>
-      <c r="V200" s="126"/>
+      <c r="V200" s="134"/>
       <c r="W200" s="2"/>
       <c r="X200" s="2"/>
       <c r="Y200" s="2"/>
@@ -9326,25 +9384,25 @@
       <c r="M201" s="104"/>
       <c r="N201" s="31"/>
       <c r="O201" s="77" t="s">
+        <v>203</v>
+      </c>
+      <c r="P201" s="76" t="s">
         <v>204</v>
       </c>
-      <c r="P201" s="76" t="s">
-        <v>205</v>
-      </c>
       <c r="Q201" s="105" t="s">
+        <v>203</v>
+      </c>
+      <c r="R201" s="76" t="s">
         <v>204</v>
       </c>
-      <c r="R201" s="76" t="s">
-        <v>205</v>
-      </c>
       <c r="S201" s="105" t="s">
+        <v>203</v>
+      </c>
+      <c r="T201" s="76" t="s">
         <v>204</v>
       </c>
-      <c r="T201" s="76" t="s">
-        <v>205</v>
-      </c>
-      <c r="U201" s="127"/>
-      <c r="V201" s="128"/>
+      <c r="U201" s="136"/>
+      <c r="V201" s="129"/>
       <c r="W201" s="2"/>
       <c r="X201" s="2"/>
       <c r="Y201" s="2"/>
@@ -9359,10 +9417,10 @@
       <c r="A202" s="2"/>
       <c r="B202" s="4"/>
       <c r="C202" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D202" s="2" t="s">
         <v>206</v>
-      </c>
-      <c r="D202" s="2" t="s">
-        <v>207</v>
       </c>
       <c r="E202" s="2"/>
       <c r="F202" s="2"/>
@@ -9562,7 +9620,7 @@
       <c r="B206" s="2"/>
       <c r="C206" s="2"/>
       <c r="D206" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E206" s="2">
         <v>2500</v>
@@ -9575,7 +9633,7 @@
       <c r="K206" s="2"/>
       <c r="L206" s="2"/>
       <c r="M206" s="70" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="N206" s="74"/>
       <c r="O206" s="74"/>
@@ -11319,7 +11377,7 @@
       <c r="A259" s="2"/>
       <c r="B259" s="2"/>
       <c r="C259" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D259" s="2"/>
       <c r="E259" s="117">
@@ -11356,7 +11414,7 @@
       <c r="A260" s="2"/>
       <c r="B260" s="2"/>
       <c r="C260" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D260" s="2"/>
       <c r="E260" s="117"/>
@@ -12442,6 +12500,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="U200:V201"/>
+    <mergeCell ref="C79:K79"/>
+    <mergeCell ref="C82:K82"/>
+    <mergeCell ref="B184:K184"/>
+    <mergeCell ref="O200:P200"/>
+    <mergeCell ref="Q200:R200"/>
+    <mergeCell ref="S200:T200"/>
     <mergeCell ref="G31:H31"/>
     <mergeCell ref="I31:J31"/>
     <mergeCell ref="B12:K12"/>
@@ -12449,13 +12514,6 @@
     <mergeCell ref="I29:J29"/>
     <mergeCell ref="G30:H30"/>
     <mergeCell ref="I30:J30"/>
-    <mergeCell ref="U200:V201"/>
-    <mergeCell ref="C79:K79"/>
-    <mergeCell ref="C82:K82"/>
-    <mergeCell ref="B184:K184"/>
-    <mergeCell ref="O200:P200"/>
-    <mergeCell ref="Q200:R200"/>
-    <mergeCell ref="S200:T200"/>
   </mergeCells>
   <conditionalFormatting sqref="E262:F262">
     <cfRule type="expression" priority="1" stopIfTrue="1">
@@ -12472,16 +12530,16 @@
           <controlPr defaultSize="0" r:id="rId4">
             <anchor moveWithCells="1">
               <from>
-                <xdr:col>4</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>594360</xdr:colOff>
                 <xdr:row>194</xdr:row>
-                <xdr:rowOff>160020</xdr:rowOff>
+                <xdr:rowOff>175260</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>4</xdr:col>
-                <xdr:colOff>289560</xdr:colOff>
+                <xdr:colOff>175260</xdr:colOff>
                 <xdr:row>196</xdr:row>
-                <xdr:rowOff>68580</xdr:rowOff>
+                <xdr:rowOff>83820</xdr:rowOff>
               </to>
             </anchor>
           </controlPr>

</xml_diff>

<commit_message>
improve and bug fixex
</commit_message>
<xml_diff>
--- a/OIC DOCS/dummy.xlsx
+++ b/OIC DOCS/dummy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev\Code\FastAPI\pc\uiic_automation\OIC DOCS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jadav\Coding\Automation\UIIC\uiic_automation\OIC DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE4F59EC-2CEC-43B5-B06D-7FAC66507F25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E86E18-178E-485C-9405-7C1D21E7DE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="254">
   <si>
     <t>Er. SUNIL KUMAR</t>
   </si>
@@ -794,6 +794,9 @@
   </si>
   <si>
     <t>compulsory_excess</t>
+  </si>
+  <si>
+    <t>jumper</t>
   </si>
 </sst>
 </file>
@@ -1631,12 +1634,39 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1655,9 +1685,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1667,32 +1694,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2000,33 +2003,33 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AE294"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.109375" style="3" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="31" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="31" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="5"/>
       <c r="C2" s="4"/>
@@ -2059,7 +2062,7 @@
       <c r="AD2" s="4"/>
       <c r="AE2" s="4"/>
     </row>
-    <row r="3" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" s="8" t="s">
         <v>0</v>
@@ -2096,7 +2099,7 @@
       <c r="AD3" s="4"/>
       <c r="AE3" s="4"/>
     </row>
-    <row r="4" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="5" t="s">
         <v>2</v>
@@ -2133,7 +2136,7 @@
       <c r="AD4" s="4"/>
       <c r="AE4" s="4"/>
     </row>
-    <row r="5" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="5" t="s">
         <v>4</v>
@@ -2170,7 +2173,7 @@
       <c r="AD5" s="4"/>
       <c r="AE5" s="4"/>
     </row>
-    <row r="6" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="11" t="s">
         <v>6</v>
@@ -2207,7 +2210,7 @@
       <c r="AD6" s="4"/>
       <c r="AE6" s="4"/>
     </row>
-    <row r="7" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="15"/>
       <c r="C7" s="16"/>
@@ -2240,7 +2243,7 @@
       <c r="AD7" s="4"/>
       <c r="AE7" s="4"/>
     </row>
-    <row r="8" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
@@ -2273,7 +2276,7 @@
       <c r="AD8" s="4"/>
       <c r="AE8" s="4"/>
     </row>
-    <row r="9" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="19" t="s">
         <v>8</v>
@@ -2312,7 +2315,7 @@
       <c r="AD9" s="4"/>
       <c r="AE9" s="4"/>
     </row>
-    <row r="10" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="19"/>
       <c r="C10" s="4"/>
@@ -2345,7 +2348,7 @@
       <c r="AD10" s="4"/>
       <c r="AE10" s="4"/>
     </row>
-    <row r="11" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="22" t="s">
         <v>11</v>
@@ -2380,20 +2383,20 @@
       <c r="AD11" s="4"/>
       <c r="AE11" s="4"/>
     </row>
-    <row r="12" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
-      <c r="B12" s="168" t="s">
+      <c r="B12" s="151" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="167"/>
-      <c r="D12" s="163"/>
-      <c r="E12" s="164"/>
-      <c r="F12" s="165"/>
-      <c r="G12" s="165"/>
-      <c r="H12" s="164"/>
-      <c r="I12" s="164"/>
-      <c r="J12" s="164"/>
-      <c r="K12" s="165"/>
+      <c r="C12" s="152"/>
+      <c r="D12" s="153"/>
+      <c r="E12" s="154"/>
+      <c r="F12" s="155"/>
+      <c r="G12" s="155"/>
+      <c r="H12" s="154"/>
+      <c r="I12" s="154"/>
+      <c r="J12" s="154"/>
+      <c r="K12" s="155"/>
       <c r="L12" s="4"/>
       <c r="M12" s="5"/>
       <c r="N12" s="7"/>
@@ -2415,7 +2418,7 @@
       <c r="AD12" s="4"/>
       <c r="AE12" s="4"/>
     </row>
-    <row r="13" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="5">
         <v>1</v>
@@ -2450,7 +2453,7 @@
       <c r="AD13" s="4"/>
       <c r="AE13" s="4"/>
     </row>
-    <row r="14" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="19" t="s">
         <v>13</v>
@@ -2495,7 +2498,7 @@
       <c r="AD14" s="4"/>
       <c r="AE14" s="4"/>
     </row>
-    <row r="15" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="25"/>
       <c r="B15" s="5"/>
       <c r="C15" s="4" t="s">
@@ -2532,7 +2535,7 @@
       <c r="AD15" s="4"/>
       <c r="AE15" s="4"/>
     </row>
-    <row r="16" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="5"/>
       <c r="C16" s="4"/>
@@ -2565,7 +2568,7 @@
       <c r="AD16" s="4"/>
       <c r="AE16" s="4"/>
     </row>
-    <row r="17" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="5" t="s">
         <v>19</v>
@@ -2614,7 +2617,7 @@
       <c r="AD17" s="4"/>
       <c r="AE17" s="4"/>
     </row>
-    <row r="18" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="5"/>
       <c r="C18" s="4"/>
@@ -2647,7 +2650,7 @@
       <c r="AD18" s="4"/>
       <c r="AE18" s="4"/>
     </row>
-    <row r="19" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="19" t="s">
         <v>24</v>
@@ -2688,7 +2691,7 @@
       <c r="AD19" s="4"/>
       <c r="AE19" s="4"/>
     </row>
-    <row r="20" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="9"/>
       <c r="B20" s="5"/>
       <c r="C20" s="4" t="s">
@@ -2727,7 +2730,7 @@
       <c r="AD20" s="4"/>
       <c r="AE20" s="4"/>
     </row>
-    <row r="21" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9"/>
       <c r="B21" s="5"/>
       <c r="C21" s="4" t="s">
@@ -2766,7 +2769,7 @@
       <c r="AD21" s="4"/>
       <c r="AE21" s="4"/>
     </row>
-    <row r="22" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9"/>
       <c r="B22" s="19"/>
       <c r="C22" s="4"/>
@@ -2803,7 +2806,7 @@
       <c r="AD22" s="4"/>
       <c r="AE22" s="4"/>
     </row>
-    <row r="23" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="19" t="s">
         <v>30</v>
@@ -2844,7 +2847,7 @@
       <c r="AD23" s="4"/>
       <c r="AE23" s="4"/>
     </row>
-    <row r="24" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9"/>
       <c r="B24" s="19"/>
       <c r="C24" s="4"/>
@@ -2877,7 +2880,7 @@
       <c r="AD24" s="4"/>
       <c r="AE24" s="4"/>
     </row>
-    <row r="25" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="19">
         <v>2</v>
@@ -2918,7 +2921,7 @@
       <c r="AD25" s="4"/>
       <c r="AE25" s="4"/>
     </row>
-    <row r="26" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="5" t="s">
         <v>13</v>
@@ -2959,7 +2962,7 @@
       <c r="AD26" s="4"/>
       <c r="AE26" s="4"/>
     </row>
-    <row r="27" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="5" t="s">
         <v>19</v>
@@ -3000,7 +3003,7 @@
       <c r="AD27" s="4"/>
       <c r="AE27" s="4"/>
     </row>
-    <row r="28" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="5" t="s">
         <v>24</v>
@@ -3041,21 +3044,21 @@
       <c r="AD28" s="4"/>
       <c r="AE28" s="4"/>
     </row>
-    <row r="29" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="5"/>
       <c r="C29" s="27"/>
       <c r="D29" s="28"/>
       <c r="E29" s="29"/>
       <c r="F29" s="30"/>
-      <c r="G29" s="159" t="s">
+      <c r="G29" s="156" t="s">
         <v>41</v>
       </c>
-      <c r="H29" s="152"/>
-      <c r="I29" s="169" t="s">
+      <c r="H29" s="157"/>
+      <c r="I29" s="158" t="s">
         <v>42</v>
       </c>
-      <c r="J29" s="152"/>
+      <c r="J29" s="157"/>
       <c r="K29" s="31" t="s">
         <v>43</v>
       </c>
@@ -3080,7 +3083,7 @@
       <c r="AD29" s="4"/>
       <c r="AE29" s="4"/>
     </row>
-    <row r="30" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
       <c r="B30" s="5" t="s">
         <v>30</v>
@@ -3093,15 +3096,15 @@
       <c r="F30" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="G30" s="170" t="s">
+      <c r="G30" s="159" t="s">
         <v>45</v>
       </c>
-      <c r="H30" s="171"/>
-      <c r="I30" s="169" t="str">
+      <c r="H30" s="160"/>
+      <c r="I30" s="158" t="str">
         <f>G30</f>
         <v>MEXC19606KT080595</v>
       </c>
-      <c r="J30" s="152"/>
+      <c r="J30" s="157"/>
       <c r="K30" s="31" t="str">
         <f>G30</f>
         <v>MEXC19606KT080595</v>
@@ -3127,7 +3130,7 @@
       <c r="AD30" s="4"/>
       <c r="AE30" s="4"/>
     </row>
-    <row r="31" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" s="5" t="s">
         <v>46</v>
@@ -3140,15 +3143,15 @@
       <c r="F31" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="G31" s="159" t="s">
+      <c r="G31" s="156" t="s">
         <v>48</v>
       </c>
-      <c r="H31" s="152"/>
-      <c r="I31" s="160" t="str">
+      <c r="H31" s="157"/>
+      <c r="I31" s="168" t="str">
         <f>G31</f>
         <v>CBZL12533</v>
       </c>
-      <c r="J31" s="161"/>
+      <c r="J31" s="169"/>
       <c r="K31" s="37" t="str">
         <f>G31</f>
         <v>CBZL12533</v>
@@ -3174,7 +3177,7 @@
       <c r="AD31" s="4"/>
       <c r="AE31" s="4"/>
     </row>
-    <row r="32" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4"/>
       <c r="B32" s="5" t="s">
         <v>49</v>
@@ -3219,7 +3222,7 @@
       <c r="AD32" s="4"/>
       <c r="AE32" s="4"/>
     </row>
-    <row r="33" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4"/>
       <c r="B33" s="5" t="s">
         <v>52</v>
@@ -3264,7 +3267,7 @@
       <c r="AD33" s="4"/>
       <c r="AE33" s="4"/>
     </row>
-    <row r="34" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4"/>
       <c r="B34" s="5" t="s">
         <v>55</v>
@@ -3309,7 +3312,7 @@
       <c r="AD34" s="4"/>
       <c r="AE34" s="4"/>
     </row>
-    <row r="35" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" s="5" t="s">
         <v>58</v>
@@ -3354,7 +3357,7 @@
       <c r="AD35" s="4"/>
       <c r="AE35" s="4"/>
     </row>
-    <row r="36" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
       <c r="B36" s="5" t="s">
         <v>61</v>
@@ -3399,7 +3402,7 @@
       <c r="AD36" s="4"/>
       <c r="AE36" s="4"/>
     </row>
-    <row r="37" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4"/>
       <c r="B37" s="5" t="s">
         <v>63</v>
@@ -3444,7 +3447,7 @@
       <c r="AD37" s="4"/>
       <c r="AE37" s="4"/>
     </row>
-    <row r="38" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4"/>
       <c r="B38" s="5" t="s">
         <v>65</v>
@@ -3489,7 +3492,7 @@
       <c r="AD38" s="4"/>
       <c r="AE38" s="4"/>
     </row>
-    <row r="39" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="5"/>
       <c r="C39" s="4" t="s">
@@ -3528,7 +3531,7 @@
       <c r="AD39" s="4"/>
       <c r="AE39" s="4"/>
     </row>
-    <row r="40" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="5"/>
       <c r="C40" s="4" t="s">
@@ -3575,7 +3578,7 @@
       <c r="AD40" s="4"/>
       <c r="AE40" s="4"/>
     </row>
-    <row r="41" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="5"/>
       <c r="C41" s="4" t="s">
@@ -3618,7 +3621,7 @@
       <c r="AD41" s="4"/>
       <c r="AE41" s="4"/>
     </row>
-    <row r="42" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="5"/>
       <c r="C42" s="4" t="s">
@@ -3661,7 +3664,7 @@
       <c r="AD42" s="4"/>
       <c r="AE42" s="4"/>
     </row>
-    <row r="43" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
       <c r="B43" s="5" t="s">
         <v>73</v>
@@ -3702,7 +3705,7 @@
       <c r="AD43" s="4"/>
       <c r="AE43" s="4"/>
     </row>
-    <row r="44" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4"/>
       <c r="B44" s="5" t="s">
         <v>75</v>
@@ -3745,7 +3748,7 @@
       <c r="AD44" s="4"/>
       <c r="AE44" s="4"/>
     </row>
-    <row r="45" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4"/>
       <c r="B45" s="5" t="s">
         <v>79</v>
@@ -3790,7 +3793,7 @@
       <c r="AD45" s="4"/>
       <c r="AE45" s="4"/>
     </row>
-    <row r="46" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4"/>
       <c r="B46" s="5" t="s">
         <v>84</v>
@@ -3829,7 +3832,7 @@
       <c r="AD46" s="4"/>
       <c r="AE46" s="4"/>
     </row>
-    <row r="47" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4"/>
       <c r="B47" s="19">
         <v>3</v>
@@ -3870,7 +3873,7 @@
       <c r="AD47" s="4"/>
       <c r="AE47" s="4"/>
     </row>
-    <row r="48" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4"/>
       <c r="B48" s="5" t="s">
         <v>13</v>
@@ -3919,7 +3922,7 @@
       <c r="AD48" s="4"/>
       <c r="AE48" s="4"/>
     </row>
-    <row r="49" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4"/>
       <c r="B49" s="5"/>
       <c r="C49" s="4" t="s">
@@ -3958,7 +3961,7 @@
       <c r="AD49" s="4"/>
       <c r="AE49" s="4"/>
     </row>
-    <row r="50" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4"/>
       <c r="B50" s="5"/>
       <c r="C50" s="4" t="s">
@@ -3997,7 +4000,7 @@
       <c r="AD50" s="4"/>
       <c r="AE50" s="4"/>
     </row>
-    <row r="51" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4"/>
       <c r="B51" s="5" t="s">
         <v>19</v>
@@ -4040,7 +4043,7 @@
       <c r="AD51" s="4"/>
       <c r="AE51" s="4"/>
     </row>
-    <row r="52" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4"/>
       <c r="B52" s="5" t="s">
         <v>24</v>
@@ -4081,7 +4084,7 @@
       <c r="AD52" s="4"/>
       <c r="AE52" s="4"/>
     </row>
-    <row r="53" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4"/>
       <c r="B53" s="5" t="s">
         <v>30</v>
@@ -4122,7 +4125,7 @@
       <c r="AD53" s="4"/>
       <c r="AE53" s="4"/>
     </row>
-    <row r="54" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4"/>
       <c r="B54" s="5" t="s">
         <v>46</v>
@@ -4167,7 +4170,7 @@
       <c r="AD54" s="4"/>
       <c r="AE54" s="4"/>
     </row>
-    <row r="55" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="4"/>
       <c r="B55" s="5" t="s">
         <v>49</v>
@@ -4208,7 +4211,7 @@
       <c r="AD55" s="4"/>
       <c r="AE55" s="4"/>
     </row>
-    <row r="56" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4"/>
       <c r="B56" s="5"/>
       <c r="C56" s="4"/>
@@ -4245,7 +4248,7 @@
       <c r="AD56" s="4"/>
       <c r="AE56" s="4"/>
     </row>
-    <row r="57" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4"/>
       <c r="B57" s="19">
         <v>4</v>
@@ -4286,7 +4289,7 @@
       <c r="AD57" s="4"/>
       <c r="AE57" s="4"/>
     </row>
-    <row r="58" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4"/>
       <c r="B58" s="5" t="s">
         <v>13</v>
@@ -4327,7 +4330,7 @@
       <c r="AD58" s="4"/>
       <c r="AE58" s="4"/>
     </row>
-    <row r="59" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4"/>
       <c r="B59" s="5" t="s">
         <v>19</v>
@@ -4368,7 +4371,7 @@
       <c r="AD59" s="4"/>
       <c r="AE59" s="4"/>
     </row>
-    <row r="60" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4"/>
       <c r="B60" s="5"/>
       <c r="C60" s="4"/>
@@ -4405,7 +4408,7 @@
       <c r="AD60" s="4"/>
       <c r="AE60" s="4"/>
     </row>
-    <row r="61" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4"/>
       <c r="B61" s="19">
         <v>5</v>
@@ -4446,7 +4449,7 @@
       <c r="AD61" s="4"/>
       <c r="AE61" s="4"/>
     </row>
-    <row r="62" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4"/>
       <c r="B62" s="5"/>
       <c r="C62" s="4" t="s">
@@ -4489,7 +4492,7 @@
       <c r="AD62" s="4"/>
       <c r="AE62" s="4"/>
     </row>
-    <row r="63" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4"/>
       <c r="B63" s="5"/>
       <c r="C63" s="4" t="s">
@@ -4534,7 +4537,7 @@
       <c r="AD63" s="4"/>
       <c r="AE63" s="4"/>
     </row>
-    <row r="64" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4"/>
       <c r="B64" s="5"/>
       <c r="C64" s="4" t="s">
@@ -4573,7 +4576,7 @@
       <c r="AD64" s="4"/>
       <c r="AE64" s="4"/>
     </row>
-    <row r="65" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4"/>
       <c r="B65" s="5"/>
       <c r="C65" s="4" t="s">
@@ -4612,7 +4615,7 @@
       <c r="AD65" s="4"/>
       <c r="AE65" s="4"/>
     </row>
-    <row r="66" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4"/>
       <c r="B66" s="5"/>
       <c r="C66" s="4"/>
@@ -4645,7 +4648,7 @@
       <c r="AD66" s="4"/>
       <c r="AE66" s="4"/>
     </row>
-    <row r="67" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="4"/>
       <c r="B67" s="5"/>
       <c r="C67" s="4"/>
@@ -4678,7 +4681,7 @@
       <c r="AD67" s="4"/>
       <c r="AE67" s="4"/>
     </row>
-    <row r="68" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4"/>
       <c r="B68" s="19">
         <v>6</v>
@@ -4715,7 +4718,7 @@
       <c r="AD68" s="4"/>
       <c r="AE68" s="4"/>
     </row>
-    <row r="69" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4"/>
       <c r="B69" s="19"/>
       <c r="C69" s="4" t="s">
@@ -4758,7 +4761,7 @@
       <c r="AD69" s="4"/>
       <c r="AE69" s="4"/>
     </row>
-    <row r="70" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4"/>
       <c r="B70" s="19"/>
       <c r="C70" s="4" t="s">
@@ -4797,7 +4800,7 @@
       <c r="AD70" s="4"/>
       <c r="AE70" s="4"/>
     </row>
-    <row r="71" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="4"/>
       <c r="B71" s="19"/>
       <c r="C71" s="4" t="s">
@@ -4836,7 +4839,7 @@
       <c r="AD71" s="4"/>
       <c r="AE71" s="4"/>
     </row>
-    <row r="72" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="4"/>
       <c r="B72" s="5"/>
       <c r="C72" s="4" t="s">
@@ -4873,7 +4876,7 @@
       <c r="AD72" s="4"/>
       <c r="AE72" s="4"/>
     </row>
-    <row r="73" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
       <c r="B73" s="19">
         <v>7</v>
@@ -4914,7 +4917,7 @@
       <c r="AD73" s="4"/>
       <c r="AE73" s="4"/>
     </row>
-    <row r="74" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4"/>
       <c r="B74" s="19"/>
       <c r="C74" s="9"/>
@@ -4947,7 +4950,7 @@
       <c r="AD74" s="4"/>
       <c r="AE74" s="4"/>
     </row>
-    <row r="75" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
       <c r="B75" s="19">
         <v>8</v>
@@ -4988,7 +4991,7 @@
       <c r="AD75" s="4"/>
       <c r="AE75" s="4"/>
     </row>
-    <row r="76" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4"/>
       <c r="B76" s="5"/>
       <c r="C76" s="4"/>
@@ -5021,7 +5024,7 @@
       <c r="AD76" s="4"/>
       <c r="AE76" s="4"/>
     </row>
-    <row r="77" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4"/>
       <c r="B77" s="19">
         <v>9</v>
@@ -5058,7 +5061,7 @@
       <c r="AD77" s="4"/>
       <c r="AE77" s="4"/>
     </row>
-    <row r="78" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
       <c r="B78" s="19"/>
       <c r="C78" s="4" t="s">
@@ -5093,20 +5096,20 @@
       <c r="AD78" s="4"/>
       <c r="AE78" s="4"/>
     </row>
-    <row r="79" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4"/>
       <c r="B79" s="19"/>
-      <c r="C79" s="162" t="s">
+      <c r="C79" s="170" t="s">
         <v>16</v>
       </c>
-      <c r="D79" s="163"/>
-      <c r="E79" s="164"/>
-      <c r="F79" s="165"/>
-      <c r="G79" s="165"/>
-      <c r="H79" s="164"/>
-      <c r="I79" s="164"/>
-      <c r="J79" s="164"/>
-      <c r="K79" s="165"/>
+      <c r="D79" s="153"/>
+      <c r="E79" s="154"/>
+      <c r="F79" s="155"/>
+      <c r="G79" s="155"/>
+      <c r="H79" s="154"/>
+      <c r="I79" s="154"/>
+      <c r="J79" s="154"/>
+      <c r="K79" s="155"/>
       <c r="L79" s="4"/>
       <c r="M79" s="5"/>
       <c r="N79" s="7"/>
@@ -5128,7 +5131,7 @@
       <c r="AD79" s="4"/>
       <c r="AE79" s="4"/>
     </row>
-    <row r="80" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
       <c r="B80" s="5"/>
       <c r="C80" s="4"/>
@@ -5165,7 +5168,7 @@
       <c r="AD80" s="4"/>
       <c r="AE80" s="4"/>
     </row>
-    <row r="81" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4"/>
       <c r="B81" s="19">
         <v>10</v>
@@ -5206,20 +5209,20 @@
       <c r="AD81" s="4"/>
       <c r="AE81" s="4"/>
     </row>
-    <row r="82" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4"/>
       <c r="B82" s="19"/>
-      <c r="C82" s="162" t="s">
+      <c r="C82" s="170" t="s">
         <v>147</v>
       </c>
-      <c r="D82" s="163"/>
-      <c r="E82" s="164"/>
-      <c r="F82" s="165"/>
-      <c r="G82" s="165"/>
-      <c r="H82" s="164"/>
-      <c r="I82" s="164"/>
-      <c r="J82" s="164"/>
-      <c r="K82" s="165"/>
+      <c r="D82" s="153"/>
+      <c r="E82" s="154"/>
+      <c r="F82" s="155"/>
+      <c r="G82" s="155"/>
+      <c r="H82" s="154"/>
+      <c r="I82" s="154"/>
+      <c r="J82" s="154"/>
+      <c r="K82" s="155"/>
       <c r="L82" s="4"/>
       <c r="M82" s="5"/>
       <c r="N82" s="7"/>
@@ -5241,7 +5244,7 @@
       <c r="AD82" s="4"/>
       <c r="AE82" s="4"/>
     </row>
-    <row r="83" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="48"/>
       <c r="B83" s="5"/>
       <c r="C83" s="4"/>
@@ -5274,7 +5277,7 @@
       <c r="AD83" s="4"/>
       <c r="AE83" s="4"/>
     </row>
-    <row r="84" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="4"/>
       <c r="B84" s="19">
         <v>11</v>
@@ -5311,7 +5314,7 @@
       <c r="AD84" s="4"/>
       <c r="AE84" s="4"/>
     </row>
-    <row r="85" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4"/>
       <c r="B85" s="19"/>
       <c r="C85" s="4" t="s">
@@ -5346,7 +5349,7 @@
       <c r="AD85" s="4"/>
       <c r="AE85" s="4"/>
     </row>
-    <row r="86" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="4"/>
       <c r="B86" s="19"/>
       <c r="C86" s="4"/>
@@ -5379,7 +5382,7 @@
       <c r="AD86" s="4"/>
       <c r="AE86" s="4"/>
     </row>
-    <row r="87" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4"/>
       <c r="B87" s="19">
         <v>12</v>
@@ -5416,7 +5419,7 @@
       <c r="AD87" s="4"/>
       <c r="AE87" s="4"/>
     </row>
-    <row r="88" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="4"/>
       <c r="B88" s="38">
         <v>1</v>
@@ -5453,7 +5456,7 @@
       <c r="AD88" s="4"/>
       <c r="AE88" s="4"/>
     </row>
-    <row r="89" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="4"/>
       <c r="B89" s="38">
         <v>2</v>
@@ -5494,7 +5497,7 @@
       <c r="AD89" s="4"/>
       <c r="AE89" s="4"/>
     </row>
-    <row r="90" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="4"/>
       <c r="B90" s="38">
         <v>3</v>
@@ -5535,7 +5538,7 @@
       <c r="AD90" s="4"/>
       <c r="AE90" s="4"/>
     </row>
-    <row r="91" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="4"/>
       <c r="B91" s="38">
         <v>4</v>
@@ -5576,7 +5579,7 @@
       <c r="AD91" s="4"/>
       <c r="AE91" s="4"/>
     </row>
-    <row r="92" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4"/>
       <c r="B92" s="38"/>
       <c r="C92" s="9"/>
@@ -5609,7 +5612,7 @@
       <c r="AD92" s="4"/>
       <c r="AE92" s="4"/>
     </row>
-    <row r="93" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="4"/>
       <c r="B93" s="19">
         <v>13</v>
@@ -5646,7 +5649,7 @@
       <c r="AD93" s="4"/>
       <c r="AE93" s="4"/>
     </row>
-    <row r="94" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="4"/>
       <c r="B94" s="19"/>
       <c r="C94" s="4"/>
@@ -5679,7 +5682,7 @@
       <c r="AD94" s="4"/>
       <c r="AE94" s="4"/>
     </row>
-    <row r="95" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="4"/>
       <c r="B95" s="49"/>
       <c r="C95" s="50"/>
@@ -5716,7 +5719,7 @@
       <c r="AD95" s="4"/>
       <c r="AE95" s="4"/>
     </row>
-    <row r="96" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="4"/>
       <c r="B96" s="55" t="s">
         <v>159</v>
@@ -5759,7 +5762,7 @@
       <c r="AD96" s="4"/>
       <c r="AE96" s="4"/>
     </row>
-    <row r="97" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="4"/>
       <c r="B97" s="49" t="s">
         <v>161</v>
@@ -5800,7 +5803,7 @@
       <c r="AD97" s="4"/>
       <c r="AE97" s="4"/>
     </row>
-    <row r="98" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="4"/>
       <c r="B98" s="59"/>
       <c r="C98" s="60"/>
@@ -5833,7 +5836,7 @@
       <c r="AD98" s="4"/>
       <c r="AE98" s="4"/>
     </row>
-    <row r="99" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="4"/>
       <c r="B99" s="11"/>
       <c r="C99" s="12"/>
@@ -5872,7 +5875,7 @@
       <c r="AD99" s="4"/>
       <c r="AE99" s="4"/>
     </row>
-    <row r="100" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="4"/>
       <c r="B100" s="63" t="s">
         <v>164</v>
@@ -5921,7 +5924,7 @@
       <c r="AD100" s="4"/>
       <c r="AE100" s="4"/>
     </row>
-    <row r="101" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="4"/>
       <c r="B101" s="33">
         <v>1</v>
@@ -5964,7 +5967,7 @@
       <c r="AD101" s="4"/>
       <c r="AE101" s="4"/>
     </row>
-    <row r="102" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="4"/>
       <c r="B102" s="73">
         <v>2</v>
@@ -6007,7 +6010,7 @@
       <c r="AD102" s="4"/>
       <c r="AE102" s="4"/>
     </row>
-    <row r="103" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="4"/>
       <c r="B103" s="73">
         <v>3</v>
@@ -6050,7 +6053,7 @@
       <c r="AD103" s="4"/>
       <c r="AE103" s="4"/>
     </row>
-    <row r="104" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="4"/>
       <c r="B104" s="73">
         <v>4</v>
@@ -6093,7 +6096,7 @@
       <c r="AD104" s="4"/>
       <c r="AE104" s="4"/>
     </row>
-    <row r="105" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="4"/>
       <c r="B105" s="73">
         <v>5</v>
@@ -6136,7 +6139,7 @@
       <c r="AD105" s="4"/>
       <c r="AE105" s="4"/>
     </row>
-    <row r="106" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="4"/>
       <c r="B106" s="73">
         <v>6</v>
@@ -6179,7 +6182,7 @@
       <c r="AD106" s="4"/>
       <c r="AE106" s="4"/>
     </row>
-    <row r="107" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="4"/>
       <c r="B107" s="73">
         <v>7</v>
@@ -6222,7 +6225,7 @@
       <c r="AD107" s="4"/>
       <c r="AE107" s="4"/>
     </row>
-    <row r="108" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="4"/>
       <c r="B108" s="73">
         <v>8</v>
@@ -6265,7 +6268,7 @@
       <c r="AD108" s="4"/>
       <c r="AE108" s="4"/>
     </row>
-    <row r="109" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="4"/>
       <c r="B109" s="73">
         <v>9</v>
@@ -6308,7 +6311,7 @@
       <c r="AD109" s="4"/>
       <c r="AE109" s="4"/>
     </row>
-    <row r="110" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="4"/>
       <c r="B110" s="73">
         <v>10</v>
@@ -6351,7 +6354,7 @@
       <c r="AD110" s="4"/>
       <c r="AE110" s="4"/>
     </row>
-    <row r="111" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="4"/>
       <c r="B111" s="73">
         <v>11</v>
@@ -6394,7 +6397,7 @@
       <c r="AD111" s="4"/>
       <c r="AE111" s="4"/>
     </row>
-    <row r="112" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="4"/>
       <c r="B112" s="73">
         <v>12</v>
@@ -6437,7 +6440,7 @@
       <c r="AD112" s="4"/>
       <c r="AE112" s="4"/>
     </row>
-    <row r="113" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="4"/>
       <c r="B113" s="73">
         <v>13</v>
@@ -6480,7 +6483,7 @@
       <c r="AD113" s="4"/>
       <c r="AE113" s="4"/>
     </row>
-    <row r="114" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="4"/>
       <c r="B114" s="73">
         <v>14</v>
@@ -6523,7 +6526,7 @@
       <c r="AD114" s="4"/>
       <c r="AE114" s="4"/>
     </row>
-    <row r="115" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="4"/>
       <c r="B115" s="73">
         <v>15</v>
@@ -6566,7 +6569,7 @@
       <c r="AD115" s="4"/>
       <c r="AE115" s="4"/>
     </row>
-    <row r="116" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="4"/>
       <c r="B116" s="73">
         <v>16</v>
@@ -6611,7 +6614,7 @@
       <c r="AD116" s="4"/>
       <c r="AE116" s="4"/>
     </row>
-    <row r="117" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="4"/>
       <c r="B117" s="73">
         <v>17</v>
@@ -6656,15 +6659,23 @@
       <c r="AD117" s="4"/>
       <c r="AE117" s="4"/>
     </row>
-    <row r="118" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="4"/>
-      <c r="B118" s="73"/>
-      <c r="C118" s="4"/>
+      <c r="B118" s="73">
+        <v>18</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D118" s="6"/>
       <c r="E118" s="71"/>
-      <c r="F118" s="72"/>
+      <c r="F118" s="72">
+        <v>150</v>
+      </c>
       <c r="G118" s="72"/>
-      <c r="H118" s="72"/>
+      <c r="H118" s="72">
+        <v>500</v>
+      </c>
       <c r="I118" s="72"/>
       <c r="J118" s="7"/>
       <c r="K118" s="5"/>
@@ -6689,7 +6700,7 @@
       <c r="AD118" s="4"/>
       <c r="AE118" s="4"/>
     </row>
-    <row r="119" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="4"/>
       <c r="B119" s="73"/>
       <c r="C119" s="4"/>
@@ -6722,7 +6733,7 @@
       <c r="AD119" s="4"/>
       <c r="AE119" s="4"/>
     </row>
-    <row r="120" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="4"/>
       <c r="B120" s="73"/>
       <c r="C120" s="4"/>
@@ -6755,7 +6766,7 @@
       <c r="AD120" s="4"/>
       <c r="AE120" s="4"/>
     </row>
-    <row r="121" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="4"/>
       <c r="B121" s="73"/>
       <c r="C121" s="4"/>
@@ -6788,7 +6799,7 @@
       <c r="AD121" s="4"/>
       <c r="AE121" s="4"/>
     </row>
-    <row r="122" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="4"/>
       <c r="B122" s="73"/>
       <c r="C122" s="4"/>
@@ -6821,7 +6832,7 @@
       <c r="AD122" s="4"/>
       <c r="AE122" s="4"/>
     </row>
-    <row r="123" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="4"/>
       <c r="B123" s="73"/>
       <c r="C123" s="4"/>
@@ -6854,7 +6865,7 @@
       <c r="AD123" s="4"/>
       <c r="AE123" s="4"/>
     </row>
-    <row r="124" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="4"/>
       <c r="B124" s="73"/>
       <c r="C124" s="4"/>
@@ -6887,7 +6898,7 @@
       <c r="AD124" s="4"/>
       <c r="AE124" s="4"/>
     </row>
-    <row r="125" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="4"/>
       <c r="B125" s="73"/>
       <c r="C125" s="4"/>
@@ -6920,7 +6931,7 @@
       <c r="AD125" s="4"/>
       <c r="AE125" s="4"/>
     </row>
-    <row r="126" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="4"/>
       <c r="B126" s="73"/>
       <c r="C126" s="4"/>
@@ -6953,7 +6964,7 @@
       <c r="AD126" s="4"/>
       <c r="AE126" s="4"/>
     </row>
-    <row r="127" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="4"/>
       <c r="B127" s="73"/>
       <c r="C127" s="4"/>
@@ -6986,7 +6997,7 @@
       <c r="AD127" s="4"/>
       <c r="AE127" s="4"/>
     </row>
-    <row r="128" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="4"/>
       <c r="B128" s="73"/>
       <c r="C128" s="4"/>
@@ -7019,7 +7030,7 @@
       <c r="AD128" s="4"/>
       <c r="AE128" s="4"/>
     </row>
-    <row r="129" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="4"/>
       <c r="B129" s="73"/>
       <c r="C129" s="4"/>
@@ -7052,7 +7063,7 @@
       <c r="AD129" s="4"/>
       <c r="AE129" s="4"/>
     </row>
-    <row r="130" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="4"/>
       <c r="B130" s="73"/>
       <c r="C130" s="4"/>
@@ -7085,7 +7096,7 @@
       <c r="AD130" s="4"/>
       <c r="AE130" s="4"/>
     </row>
-    <row r="131" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="4"/>
       <c r="B131" s="73"/>
       <c r="C131" s="4"/>
@@ -7118,7 +7129,7 @@
       <c r="AD131" s="4"/>
       <c r="AE131" s="4"/>
     </row>
-    <row r="132" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="4"/>
       <c r="B132" s="73"/>
       <c r="C132" s="4"/>
@@ -7151,7 +7162,7 @@
       <c r="AD132" s="4"/>
       <c r="AE132" s="4"/>
     </row>
-    <row r="133" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="4"/>
       <c r="B133" s="73"/>
       <c r="C133" s="4"/>
@@ -7184,7 +7195,7 @@
       <c r="AD133" s="4"/>
       <c r="AE133" s="4"/>
     </row>
-    <row r="134" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="4"/>
       <c r="B134" s="73"/>
       <c r="C134" s="4"/>
@@ -7217,7 +7228,7 @@
       <c r="AD134" s="4"/>
       <c r="AE134" s="4"/>
     </row>
-    <row r="135" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="4"/>
       <c r="B135" s="77"/>
       <c r="C135" s="78"/>
@@ -7252,7 +7263,7 @@
       <c r="AD135" s="4"/>
       <c r="AE135" s="4"/>
     </row>
-    <row r="136" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="4"/>
       <c r="B136" s="55" t="s">
         <v>190</v>
@@ -7262,7 +7273,7 @@
       <c r="E136" s="71"/>
       <c r="F136" s="72">
         <f>SUM(F101:F135)</f>
-        <v>139226</v>
+        <v>139376</v>
       </c>
       <c r="G136" s="83">
         <f>SUM(G101:G135)</f>
@@ -7270,7 +7281,7 @@
       </c>
       <c r="H136" s="84">
         <f>SUM(H101:H135)</f>
-        <v>539</v>
+        <v>1039</v>
       </c>
       <c r="I136" s="84">
         <f>SUM(I101:I135)</f>
@@ -7302,7 +7313,7 @@
       <c r="AD136" s="4"/>
       <c r="AE136" s="4"/>
     </row>
-    <row r="137" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="85"/>
       <c r="B137" s="86">
         <v>18</v>
@@ -7314,7 +7325,7 @@
       <c r="E137" s="65"/>
       <c r="F137" s="87">
         <f>B137*F136/100</f>
-        <v>25060.68</v>
+        <v>25087.68</v>
       </c>
       <c r="G137" s="87">
         <f>B137*G136/100</f>
@@ -7322,7 +7333,7 @@
       </c>
       <c r="H137" s="87">
         <f>B137*H136/100</f>
-        <v>97.02</v>
+        <v>187.02</v>
       </c>
       <c r="I137" s="87">
         <f>18*I136/100</f>
@@ -7351,7 +7362,7 @@
       <c r="AD137" s="4"/>
       <c r="AE137" s="4"/>
     </row>
-    <row r="138" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="4"/>
       <c r="B138" s="55" t="s">
         <v>190</v>
@@ -7361,7 +7372,7 @@
       <c r="E138" s="7"/>
       <c r="F138" s="83">
         <f>SUM(F136:F137)</f>
-        <v>164286.68</v>
+        <v>164463.67999999999</v>
       </c>
       <c r="G138" s="83">
         <f>SUM(G136:G137)</f>
@@ -7369,7 +7380,7 @@
       </c>
       <c r="H138" s="83">
         <f>SUM(H136:H137)</f>
-        <v>636.02</v>
+        <v>1226.02</v>
       </c>
       <c r="I138" s="84">
         <f>SUM(I136:I137)</f>
@@ -7398,7 +7409,7 @@
       <c r="AD138" s="4"/>
       <c r="AE138" s="4"/>
     </row>
-    <row r="139" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="4"/>
       <c r="B139" s="88" t="s">
         <v>192</v>
@@ -7433,7 +7444,7 @@
       <c r="AD139" s="4"/>
       <c r="AE139" s="4"/>
     </row>
-    <row r="140" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="4"/>
       <c r="B140" s="89">
         <f>J96</f>
@@ -7451,7 +7462,7 @@
       </c>
       <c r="H140" s="90">
         <f>H138/2</f>
-        <v>318.01</v>
+        <v>613.01</v>
       </c>
       <c r="I140" s="84">
         <v>0</v>
@@ -7479,7 +7490,7 @@
       <c r="AD140" s="4"/>
       <c r="AE140" s="4"/>
     </row>
-    <row r="141" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="4"/>
       <c r="B141" s="49" t="s">
         <v>194</v>
@@ -7489,7 +7500,7 @@
       <c r="E141" s="91"/>
       <c r="F141" s="92">
         <f>F138</f>
-        <v>164286.68</v>
+        <v>164463.67999999999</v>
       </c>
       <c r="G141" s="93">
         <f>G138-G140</f>
@@ -7497,7 +7508,7 @@
       </c>
       <c r="H141" s="92">
         <f>H138-H140</f>
-        <v>318.01</v>
+        <v>613.01</v>
       </c>
       <c r="I141" s="93">
         <f>I138-I140</f>
@@ -7526,7 +7537,7 @@
       <c r="AD141" s="4"/>
       <c r="AE141" s="4"/>
     </row>
-    <row r="142" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="4"/>
       <c r="B142" s="63" t="s">
         <v>195</v>
@@ -7536,11 +7547,11 @@
       <c r="E142" s="94"/>
       <c r="F142" s="95">
         <f>F141</f>
-        <v>164286.68</v>
+        <v>164463.67999999999</v>
       </c>
       <c r="G142" s="96">
         <f>G141+H141+I141+J141</f>
-        <v>4124.8197999999993</v>
+        <v>4419.8197999999993</v>
       </c>
       <c r="H142" s="97"/>
       <c r="I142" s="91"/>
@@ -7567,7 +7578,7 @@
       <c r="AD142" s="4"/>
       <c r="AE142" s="4"/>
     </row>
-    <row r="143" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="4"/>
       <c r="B143" s="19"/>
       <c r="C143" s="4"/>
@@ -7600,7 +7611,7 @@
       <c r="AD143" s="4"/>
       <c r="AE143" s="4"/>
     </row>
-    <row r="144" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="4"/>
       <c r="B144" s="19" t="s">
         <v>196</v>
@@ -7611,7 +7622,7 @@
       <c r="F144" s="5"/>
       <c r="G144" s="20">
         <f>G140+H140+J140+I140</f>
-        <v>318.01</v>
+        <v>613.01</v>
       </c>
       <c r="H144" s="7"/>
       <c r="I144" s="7"/>
@@ -7638,7 +7649,7 @@
       <c r="AD144" s="4"/>
       <c r="AE144" s="4"/>
     </row>
-    <row r="145" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="4"/>
       <c r="B145" s="5"/>
       <c r="C145" s="4"/>
@@ -7671,7 +7682,7 @@
       <c r="AD145" s="4"/>
       <c r="AE145" s="4"/>
     </row>
-    <row r="146" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="4"/>
       <c r="B146" s="5"/>
       <c r="C146" s="4"/>
@@ -7704,7 +7715,7 @@
       <c r="AD146" s="4"/>
       <c r="AE146" s="4"/>
     </row>
-    <row r="147" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="4"/>
       <c r="B147" s="5"/>
       <c r="C147" s="4"/>
@@ -7737,7 +7748,7 @@
       <c r="AD147" s="4"/>
       <c r="AE147" s="4"/>
     </row>
-    <row r="148" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="4"/>
       <c r="B148" s="5"/>
       <c r="C148" s="4"/>
@@ -7770,7 +7781,7 @@
       <c r="AD148" s="4"/>
       <c r="AE148" s="4"/>
     </row>
-    <row r="149" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="4"/>
       <c r="B149" s="5"/>
       <c r="C149" s="4"/>
@@ -7803,7 +7814,7 @@
       <c r="AD149" s="4"/>
       <c r="AE149" s="4"/>
     </row>
-    <row r="150" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="4"/>
       <c r="B150" s="5"/>
       <c r="C150" s="4"/>
@@ -7836,7 +7847,7 @@
       <c r="AD150" s="4"/>
       <c r="AE150" s="4"/>
     </row>
-    <row r="151" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="4"/>
       <c r="B151" s="5"/>
       <c r="C151" s="4"/>
@@ -7869,7 +7880,7 @@
       <c r="AD151" s="4"/>
       <c r="AE151" s="4"/>
     </row>
-    <row r="152" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="4"/>
       <c r="B152" s="5"/>
       <c r="C152" s="4"/>
@@ -7902,7 +7913,7 @@
       <c r="AD152" s="4"/>
       <c r="AE152" s="4"/>
     </row>
-    <row r="153" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="4"/>
       <c r="B153" s="22" t="s">
         <v>197</v>
@@ -7937,7 +7948,7 @@
       <c r="AD153" s="4"/>
       <c r="AE153" s="4"/>
     </row>
-    <row r="154" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="4"/>
       <c r="B154" s="5"/>
       <c r="C154" s="4"/>
@@ -7970,7 +7981,7 @@
       <c r="AD154" s="4"/>
       <c r="AE154" s="4"/>
     </row>
-    <row r="155" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="4"/>
       <c r="B155" s="98" t="s">
         <v>198</v>
@@ -8005,7 +8016,7 @@
       <c r="AD155" s="4"/>
       <c r="AE155" s="4"/>
     </row>
-    <row r="156" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="4"/>
       <c r="B156" s="100" t="s">
         <v>164</v>
@@ -8050,7 +8061,7 @@
       <c r="AD156" s="4"/>
       <c r="AE156" s="4"/>
     </row>
-    <row r="157" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="4"/>
       <c r="B157" s="73">
         <v>1</v>
@@ -8089,7 +8100,7 @@
       <c r="AD157" s="4"/>
       <c r="AE157" s="4"/>
     </row>
-    <row r="158" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="4"/>
       <c r="B158" s="73">
         <v>2</v>
@@ -8128,7 +8139,7 @@
       <c r="AD158" s="4"/>
       <c r="AE158" s="4"/>
     </row>
-    <row r="159" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="4"/>
       <c r="B159" s="73">
         <v>3</v>
@@ -8167,7 +8178,7 @@
       <c r="AD159" s="4"/>
       <c r="AE159" s="4"/>
     </row>
-    <row r="160" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="4"/>
       <c r="B160" s="73"/>
       <c r="C160" s="4"/>
@@ -8200,7 +8211,7 @@
       <c r="AD160" s="4"/>
       <c r="AE160" s="4"/>
     </row>
-    <row r="161" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="4"/>
       <c r="B161" s="73"/>
       <c r="C161" s="4"/>
@@ -8233,7 +8244,7 @@
       <c r="AD161" s="4"/>
       <c r="AE161" s="4"/>
     </row>
-    <row r="162" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="4"/>
       <c r="B162" s="107" t="s">
         <v>190</v>
@@ -8280,7 +8291,7 @@
       <c r="AD162" s="4"/>
       <c r="AE162" s="4"/>
     </row>
-    <row r="163" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="4"/>
       <c r="B163" s="109"/>
       <c r="C163" s="12"/>
@@ -8313,7 +8324,7 @@
       <c r="AD163" s="4"/>
       <c r="AE163" s="4"/>
     </row>
-    <row r="164" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="85"/>
       <c r="B164" s="98" t="s">
         <v>190</v>
@@ -8360,7 +8371,7 @@
       <c r="AD164" s="4"/>
       <c r="AE164" s="4"/>
     </row>
-    <row r="165" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="4"/>
       <c r="B165" s="63"/>
       <c r="C165" s="12"/>
@@ -8398,7 +8409,7 @@
       <c r="AD165" s="4"/>
       <c r="AE165" s="4"/>
     </row>
-    <row r="166" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="4"/>
       <c r="B166" s="115"/>
       <c r="C166" s="60"/>
@@ -8431,7 +8442,7 @@
       <c r="AD166" s="4"/>
       <c r="AE166" s="4"/>
     </row>
-    <row r="167" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="4"/>
       <c r="B167" s="98" t="s">
         <v>208</v>
@@ -8470,7 +8481,7 @@
       <c r="AD167" s="4"/>
       <c r="AE167" s="4"/>
     </row>
-    <row r="168" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="4"/>
       <c r="B168" s="88"/>
       <c r="C168" s="4"/>
@@ -8509,7 +8520,7 @@
       <c r="AD168" s="4"/>
       <c r="AE168" s="4"/>
     </row>
-    <row r="169" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="4"/>
       <c r="B169" s="118">
         <f>J97</f>
@@ -8553,7 +8564,7 @@
       <c r="AD169" s="4"/>
       <c r="AE169" s="4"/>
     </row>
-    <row r="170" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="4"/>
       <c r="B170" s="98" t="s">
         <v>210</v>
@@ -8594,7 +8605,7 @@
       <c r="AD170" s="4"/>
       <c r="AE170" s="4"/>
     </row>
-    <row r="171" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="4"/>
       <c r="B171" s="5"/>
       <c r="C171" s="4"/>
@@ -8627,7 +8638,7 @@
       <c r="AD171" s="4"/>
       <c r="AE171" s="4"/>
     </row>
-    <row r="172" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="4"/>
       <c r="B172" s="19" t="s">
         <v>211</v>
@@ -8665,7 +8676,7 @@
       <c r="AD172" s="4"/>
       <c r="AE172" s="4"/>
     </row>
-    <row r="173" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="4"/>
       <c r="B173" s="11"/>
       <c r="C173" s="12"/>
@@ -8698,7 +8709,7 @@
       <c r="AD173" s="4"/>
       <c r="AE173" s="4"/>
     </row>
-    <row r="174" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="4"/>
       <c r="B174" s="63" t="s">
         <v>212</v>
@@ -8737,7 +8748,7 @@
       <c r="AD174" s="4"/>
       <c r="AE174" s="4"/>
     </row>
-    <row r="175" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="4"/>
       <c r="B175" s="120" t="s">
         <v>213</v>
@@ -8747,11 +8758,11 @@
       <c r="E175" s="62"/>
       <c r="F175" s="106">
         <f>F142</f>
-        <v>164286.68</v>
+        <v>164463.67999999999</v>
       </c>
       <c r="G175" s="112">
         <f>G142</f>
-        <v>4124.8197999999993</v>
+        <v>4419.8197999999993</v>
       </c>
       <c r="H175" s="7"/>
       <c r="I175" s="7"/>
@@ -8778,7 +8789,7 @@
       <c r="AD175" s="4"/>
       <c r="AE175" s="4"/>
     </row>
-    <row r="176" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="4"/>
       <c r="B176" s="109" t="s">
         <v>214</v>
@@ -8819,7 +8830,7 @@
       <c r="AD176" s="4"/>
       <c r="AE176" s="4"/>
     </row>
-    <row r="177" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="4"/>
       <c r="B177" s="55" t="s">
         <v>190</v>
@@ -8829,11 +8840,11 @@
       <c r="E177" s="71"/>
       <c r="F177" s="72">
         <f>F175+F176</f>
-        <v>164286.68</v>
+        <v>164463.67999999999</v>
       </c>
       <c r="G177" s="72">
         <f>G175+G176</f>
-        <v>4142.5197999999991</v>
+        <v>4437.5197999999991</v>
       </c>
       <c r="H177" s="7"/>
       <c r="I177" s="7"/>
@@ -8860,7 +8871,7 @@
       <c r="AD177" s="4"/>
       <c r="AE177" s="4"/>
     </row>
-    <row r="178" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="4"/>
       <c r="B178" s="109" t="s">
         <v>215</v>
@@ -8898,7 +8909,7 @@
       <c r="AD178" s="4"/>
       <c r="AE178" s="4"/>
     </row>
-    <row r="179" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="4"/>
       <c r="B179" s="63" t="s">
         <v>216</v>
@@ -8908,11 +8919,11 @@
       <c r="E179" s="94"/>
       <c r="F179" s="119">
         <f>F177</f>
-        <v>164286.68</v>
+        <v>164463.67999999999</v>
       </c>
       <c r="G179" s="121">
         <f>G177-G178</f>
-        <v>3642.5197999999991</v>
+        <v>3937.5197999999991</v>
       </c>
       <c r="H179" s="7"/>
       <c r="I179" s="7"/>
@@ -8939,7 +8950,7 @@
       <c r="AD179" s="4"/>
       <c r="AE179" s="4"/>
     </row>
-    <row r="180" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="4"/>
       <c r="B180" s="5"/>
       <c r="C180" s="4"/>
@@ -8972,7 +8983,7 @@
       <c r="AD180" s="4"/>
       <c r="AE180" s="4"/>
     </row>
-    <row r="181" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="4"/>
       <c r="B181" s="5" t="s">
         <v>217</v>
@@ -9009,7 +9020,7 @@
       <c r="AD181" s="4"/>
       <c r="AE181" s="4"/>
     </row>
-    <row r="182" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="4"/>
       <c r="B182" s="98" t="s">
         <v>218</v>
@@ -9020,7 +9031,7 @@
       <c r="F182" s="53"/>
       <c r="G182" s="68">
         <f>G179-G181</f>
-        <v>3642.5197999999991</v>
+        <v>3937.5197999999991</v>
       </c>
       <c r="H182" s="7"/>
       <c r="I182" s="56"/>
@@ -9047,7 +9058,7 @@
       <c r="AD182" s="4"/>
       <c r="AE182" s="4"/>
     </row>
-    <row r="183" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="4"/>
       <c r="B183" s="5"/>
       <c r="C183" s="4"/>
@@ -9080,20 +9091,20 @@
       <c r="AD183" s="4"/>
       <c r="AE183" s="4"/>
     </row>
-    <row r="184" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="4"/>
-      <c r="B184" s="166" t="s">
+      <c r="B184" s="171" t="s">
         <v>219</v>
       </c>
-      <c r="C184" s="167"/>
-      <c r="D184" s="163"/>
-      <c r="E184" s="164"/>
-      <c r="F184" s="165"/>
-      <c r="G184" s="165"/>
-      <c r="H184" s="164"/>
-      <c r="I184" s="164"/>
-      <c r="J184" s="164"/>
-      <c r="K184" s="165"/>
+      <c r="C184" s="152"/>
+      <c r="D184" s="153"/>
+      <c r="E184" s="154"/>
+      <c r="F184" s="155"/>
+      <c r="G184" s="155"/>
+      <c r="H184" s="154"/>
+      <c r="I184" s="154"/>
+      <c r="J184" s="154"/>
+      <c r="K184" s="155"/>
       <c r="L184" s="4"/>
       <c r="M184" s="5"/>
       <c r="N184" s="7"/>
@@ -9115,7 +9126,7 @@
       <c r="AD184" s="4"/>
       <c r="AE184" s="4"/>
     </row>
-    <row r="185" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="4"/>
       <c r="B185" s="23"/>
       <c r="C185" s="47"/>
@@ -9148,7 +9159,7 @@
       <c r="AD185" s="4"/>
       <c r="AE185" s="4"/>
     </row>
-    <row r="186" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="4"/>
       <c r="B186" s="124" t="s">
         <v>220</v>
@@ -9183,7 +9194,7 @@
       <c r="AD186" s="4"/>
       <c r="AE186" s="4"/>
     </row>
-    <row r="187" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="4"/>
       <c r="B187" s="19"/>
       <c r="C187" s="4"/>
@@ -9216,7 +9227,7 @@
       <c r="AD187" s="4"/>
       <c r="AE187" s="4"/>
     </row>
-    <row r="188" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="4"/>
       <c r="B188" s="5">
         <v>1</v>
@@ -9258,7 +9269,7 @@
       <c r="AD188" s="4"/>
       <c r="AE188" s="4"/>
     </row>
-    <row r="189" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="4"/>
       <c r="B189" s="5"/>
       <c r="C189" s="4"/>
@@ -9291,7 +9302,7 @@
       <c r="AD189" s="4"/>
       <c r="AE189" s="4"/>
     </row>
-    <row r="190" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="4"/>
       <c r="B190" s="5">
         <v>2</v>
@@ -9333,7 +9344,7 @@
       <c r="AD190" s="4"/>
       <c r="AE190" s="4"/>
     </row>
-    <row r="191" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="4"/>
       <c r="B191" s="19"/>
       <c r="C191" s="4"/>
@@ -9366,7 +9377,7 @@
       <c r="AD191" s="4"/>
       <c r="AE191" s="4"/>
     </row>
-    <row r="192" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="4"/>
       <c r="B192" s="19"/>
       <c r="C192" s="125" t="s">
@@ -9403,7 +9414,7 @@
       <c r="AD192" s="4"/>
       <c r="AE192" s="4"/>
     </row>
-    <row r="193" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="4"/>
       <c r="B193" s="5"/>
       <c r="C193" s="32"/>
@@ -9436,7 +9447,7 @@
       <c r="AD193" s="4"/>
       <c r="AE193" s="4"/>
     </row>
-    <row r="194" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="4"/>
       <c r="B194" s="19"/>
       <c r="C194" s="126" t="s">
@@ -9471,7 +9482,7 @@
       <c r="AD194" s="4"/>
       <c r="AE194" s="4"/>
     </row>
-    <row r="195" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="4"/>
       <c r="B195" s="19"/>
       <c r="C195" s="4"/>
@@ -9504,7 +9515,7 @@
       <c r="AD195" s="4"/>
       <c r="AE195" s="4"/>
     </row>
-    <row r="196" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="4"/>
       <c r="B196" s="19"/>
       <c r="C196" s="4"/>
@@ -9537,7 +9548,7 @@
       <c r="AD196" s="4"/>
       <c r="AE196" s="4"/>
     </row>
-    <row r="197" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="4"/>
       <c r="B197" s="19"/>
       <c r="C197" s="4"/>
@@ -9570,7 +9581,7 @@
       <c r="AD197" s="4"/>
       <c r="AE197" s="4"/>
     </row>
-    <row r="198" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="4"/>
       <c r="B198" s="5"/>
       <c r="C198" s="4" t="s">
@@ -9615,7 +9626,7 @@
       <c r="AD198" s="4"/>
       <c r="AE198" s="4"/>
     </row>
-    <row r="199" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="4"/>
       <c r="B199" s="5"/>
       <c r="C199" s="4"/>
@@ -9648,7 +9659,7 @@
       <c r="AD199" s="4"/>
       <c r="AE199" s="4"/>
     </row>
-    <row r="200" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="4"/>
       <c r="B200" s="5"/>
       <c r="C200" s="4"/>
@@ -9667,22 +9678,22 @@
       <c r="N200" s="130" t="s">
         <v>229</v>
       </c>
-      <c r="O200" s="151" t="s">
+      <c r="O200" s="161" t="s">
         <v>230</v>
       </c>
-      <c r="P200" s="152"/>
-      <c r="Q200" s="151" t="s">
+      <c r="P200" s="157"/>
+      <c r="Q200" s="161" t="s">
         <v>231</v>
       </c>
-      <c r="R200" s="152"/>
-      <c r="S200" s="153" t="s">
+      <c r="R200" s="157"/>
+      <c r="S200" s="162" t="s">
         <v>232</v>
       </c>
-      <c r="T200" s="154"/>
-      <c r="U200" s="155" t="s">
+      <c r="T200" s="163"/>
+      <c r="U200" s="164" t="s">
         <v>233</v>
       </c>
-      <c r="V200" s="156"/>
+      <c r="V200" s="165"/>
       <c r="W200" s="4"/>
       <c r="X200" s="4"/>
       <c r="Y200" s="4"/>
@@ -9693,7 +9704,7 @@
       <c r="AD200" s="4"/>
       <c r="AE200" s="4"/>
     </row>
-    <row r="201" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="4"/>
       <c r="B201" s="5"/>
       <c r="C201" s="4"/>
@@ -9726,8 +9737,8 @@
       <c r="T201" s="136" t="s">
         <v>235</v>
       </c>
-      <c r="U201" s="157"/>
-      <c r="V201" s="158"/>
+      <c r="U201" s="166"/>
+      <c r="V201" s="167"/>
       <c r="W201" s="4"/>
       <c r="X201" s="4"/>
       <c r="Y201" s="4"/>
@@ -9738,7 +9749,7 @@
       <c r="AD201" s="4"/>
       <c r="AE201" s="4"/>
     </row>
-    <row r="202" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A202" s="4"/>
       <c r="B202" s="19"/>
       <c r="C202" s="4" t="s">
@@ -9758,27 +9769,27 @@
       <c r="M202" s="137"/>
       <c r="N202" s="43">
         <f>G136+H136</f>
-        <v>2742.11</v>
+        <v>3242.11</v>
       </c>
       <c r="O202" s="137">
         <v>14</v>
       </c>
       <c r="P202" s="138">
         <f>14*N202/100</f>
-        <v>383.8954</v>
+        <v>453.8954</v>
       </c>
       <c r="Q202" s="139">
         <v>14</v>
       </c>
       <c r="R202" s="138">
         <f>P202</f>
-        <v>383.8954</v>
+        <v>453.8954</v>
       </c>
       <c r="S202" s="70"/>
       <c r="T202" s="85"/>
       <c r="U202" s="56">
         <f>P202+R202</f>
-        <v>767.79079999999999</v>
+        <v>907.79079999999999</v>
       </c>
       <c r="V202" s="85"/>
       <c r="W202" s="4"/>
@@ -9791,7 +9802,7 @@
       <c r="AD202" s="4"/>
       <c r="AE202" s="4"/>
     </row>
-    <row r="203" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A203" s="4"/>
       <c r="B203" s="19"/>
       <c r="C203" s="4"/>
@@ -9840,7 +9851,7 @@
       <c r="AD203" s="4"/>
       <c r="AE203" s="4"/>
     </row>
-    <row r="204" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A204" s="4"/>
       <c r="B204" s="19"/>
       <c r="C204" s="4"/>
@@ -9889,7 +9900,7 @@
       <c r="AD204" s="4"/>
       <c r="AE204" s="4"/>
     </row>
-    <row r="205" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A205" s="4"/>
       <c r="B205" s="19"/>
       <c r="C205" s="4"/>
@@ -9940,7 +9951,7 @@
       <c r="AD205" s="4"/>
       <c r="AE205" s="4"/>
     </row>
-    <row r="206" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A206" s="4"/>
       <c r="B206" s="5"/>
       <c r="C206" s="4"/>
@@ -9969,7 +9980,7 @@
       <c r="T206" s="101"/>
       <c r="U206" s="99">
         <f>SUM(U202:U205)</f>
-        <v>4873.4431999999997</v>
+        <v>5013.4431999999997</v>
       </c>
       <c r="V206" s="147"/>
       <c r="W206" s="4"/>
@@ -9982,7 +9993,7 @@
       <c r="AD206" s="4"/>
       <c r="AE206" s="4"/>
     </row>
-    <row r="207" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A207" s="4"/>
       <c r="B207" s="5"/>
       <c r="C207" s="4"/>
@@ -10015,7 +10026,7 @@
       <c r="AD207" s="4"/>
       <c r="AE207" s="4"/>
     </row>
-    <row r="208" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A208" s="4"/>
       <c r="B208" s="5"/>
       <c r="C208" s="4"/>
@@ -10048,7 +10059,7 @@
       <c r="AD208" s="4"/>
       <c r="AE208" s="4"/>
     </row>
-    <row r="209" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A209" s="4"/>
       <c r="B209" s="19"/>
       <c r="C209" s="4"/>
@@ -10081,7 +10092,7 @@
       <c r="AD209" s="4"/>
       <c r="AE209" s="4"/>
     </row>
-    <row r="210" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A210" s="4"/>
       <c r="B210" s="19"/>
       <c r="C210" s="4"/>
@@ -10114,7 +10125,7 @@
       <c r="AD210" s="4"/>
       <c r="AE210" s="4"/>
     </row>
-    <row r="211" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A211" s="4"/>
       <c r="B211" s="19"/>
       <c r="C211" s="4"/>
@@ -10147,7 +10158,7 @@
       <c r="AD211" s="4"/>
       <c r="AE211" s="4"/>
     </row>
-    <row r="212" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A212" s="4"/>
       <c r="B212" s="19"/>
       <c r="C212" s="4"/>
@@ -10180,7 +10191,7 @@
       <c r="AD212" s="4"/>
       <c r="AE212" s="4"/>
     </row>
-    <row r="213" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A213" s="4"/>
       <c r="B213" s="19"/>
       <c r="C213" s="4"/>
@@ -10213,7 +10224,7 @@
       <c r="AD213" s="4"/>
       <c r="AE213" s="4"/>
     </row>
-    <row r="214" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="4"/>
       <c r="B214" s="19"/>
       <c r="C214" s="4"/>
@@ -10246,7 +10257,7 @@
       <c r="AD214" s="4"/>
       <c r="AE214" s="4"/>
     </row>
-    <row r="215" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A215" s="4"/>
       <c r="B215" s="19"/>
       <c r="C215" s="4"/>
@@ -10279,7 +10290,7 @@
       <c r="AD215" s="4"/>
       <c r="AE215" s="4"/>
     </row>
-    <row r="216" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A216" s="4"/>
       <c r="B216" s="19"/>
       <c r="C216" s="4"/>
@@ -10312,7 +10323,7 @@
       <c r="AD216" s="4"/>
       <c r="AE216" s="4"/>
     </row>
-    <row r="217" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A217" s="4"/>
       <c r="B217" s="19"/>
       <c r="C217" s="4"/>
@@ -10345,7 +10356,7 @@
       <c r="AD217" s="4"/>
       <c r="AE217" s="4"/>
     </row>
-    <row r="218" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A218" s="4"/>
       <c r="B218" s="19"/>
       <c r="C218" s="4"/>
@@ -10378,7 +10389,7 @@
       <c r="AD218" s="4"/>
       <c r="AE218" s="4"/>
     </row>
-    <row r="219" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A219" s="4"/>
       <c r="B219" s="19"/>
       <c r="C219" s="4"/>
@@ -10411,7 +10422,7 @@
       <c r="AD219" s="4"/>
       <c r="AE219" s="4"/>
     </row>
-    <row r="220" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A220" s="4"/>
       <c r="B220" s="19"/>
       <c r="C220" s="4"/>
@@ -10444,7 +10455,7 @@
       <c r="AD220" s="4"/>
       <c r="AE220" s="4"/>
     </row>
-    <row r="221" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A221" s="4"/>
       <c r="B221" s="19"/>
       <c r="C221" s="4"/>
@@ -10477,7 +10488,7 @@
       <c r="AD221" s="4"/>
       <c r="AE221" s="4"/>
     </row>
-    <row r="222" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A222" s="4"/>
       <c r="B222" s="19"/>
       <c r="C222" s="4"/>
@@ -10510,7 +10521,7 @@
       <c r="AD222" s="4"/>
       <c r="AE222" s="4"/>
     </row>
-    <row r="223" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A223" s="4"/>
       <c r="B223" s="19"/>
       <c r="C223" s="4"/>
@@ -10543,7 +10554,7 @@
       <c r="AD223" s="4"/>
       <c r="AE223" s="4"/>
     </row>
-    <row r="224" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A224" s="4"/>
       <c r="B224" s="19"/>
       <c r="C224" s="4"/>
@@ -10576,7 +10587,7 @@
       <c r="AD224" s="4"/>
       <c r="AE224" s="4"/>
     </row>
-    <row r="225" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A225" s="4"/>
       <c r="B225" s="19"/>
       <c r="C225" s="4"/>
@@ -10609,7 +10620,7 @@
       <c r="AD225" s="4"/>
       <c r="AE225" s="4"/>
     </row>
-    <row r="226" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A226" s="4"/>
       <c r="B226" s="19"/>
       <c r="C226" s="4"/>
@@ -10642,7 +10653,7 @@
       <c r="AD226" s="4"/>
       <c r="AE226" s="4"/>
     </row>
-    <row r="227" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A227" s="4"/>
       <c r="B227" s="19"/>
       <c r="C227" s="4"/>
@@ -10675,7 +10686,7 @@
       <c r="AD227" s="4"/>
       <c r="AE227" s="4"/>
     </row>
-    <row r="228" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A228" s="4"/>
       <c r="B228" s="19"/>
       <c r="C228" s="4"/>
@@ -10708,7 +10719,7 @@
       <c r="AD228" s="4"/>
       <c r="AE228" s="4"/>
     </row>
-    <row r="229" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A229" s="4"/>
       <c r="B229" s="19"/>
       <c r="C229" s="4"/>
@@ -10741,7 +10752,7 @@
       <c r="AD229" s="4"/>
       <c r="AE229" s="4"/>
     </row>
-    <row r="230" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A230" s="4"/>
       <c r="B230" s="19"/>
       <c r="C230" s="4"/>
@@ -10774,7 +10785,7 @@
       <c r="AD230" s="4"/>
       <c r="AE230" s="4"/>
     </row>
-    <row r="231" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A231" s="4"/>
       <c r="B231" s="19"/>
       <c r="C231" s="4"/>
@@ -10807,7 +10818,7 @@
       <c r="AD231" s="4"/>
       <c r="AE231" s="4"/>
     </row>
-    <row r="232" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A232" s="4"/>
       <c r="B232" s="19"/>
       <c r="C232" s="4"/>
@@ -10840,7 +10851,7 @@
       <c r="AD232" s="4"/>
       <c r="AE232" s="4"/>
     </row>
-    <row r="233" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A233" s="4"/>
       <c r="B233" s="19"/>
       <c r="C233" s="4"/>
@@ -10873,7 +10884,7 @@
       <c r="AD233" s="4"/>
       <c r="AE233" s="4"/>
     </row>
-    <row r="234" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A234" s="4"/>
       <c r="B234" s="19"/>
       <c r="C234" s="4"/>
@@ -10906,7 +10917,7 @@
       <c r="AD234" s="4"/>
       <c r="AE234" s="4"/>
     </row>
-    <row r="235" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A235" s="4"/>
       <c r="B235" s="19"/>
       <c r="C235" s="4"/>
@@ -10939,7 +10950,7 @@
       <c r="AD235" s="4"/>
       <c r="AE235" s="4"/>
     </row>
-    <row r="236" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A236" s="4"/>
       <c r="B236" s="19"/>
       <c r="C236" s="4"/>
@@ -10972,7 +10983,7 @@
       <c r="AD236" s="4"/>
       <c r="AE236" s="4"/>
     </row>
-    <row r="237" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A237" s="4"/>
       <c r="B237" s="19"/>
       <c r="C237" s="4"/>
@@ -11005,7 +11016,7 @@
       <c r="AD237" s="4"/>
       <c r="AE237" s="4"/>
     </row>
-    <row r="238" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A238" s="4"/>
       <c r="B238" s="19"/>
       <c r="C238" s="4"/>
@@ -11038,7 +11049,7 @@
       <c r="AD238" s="4"/>
       <c r="AE238" s="4"/>
     </row>
-    <row r="239" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A239" s="4"/>
       <c r="B239" s="19"/>
       <c r="C239" s="4"/>
@@ -11071,7 +11082,7 @@
       <c r="AD239" s="4"/>
       <c r="AE239" s="4"/>
     </row>
-    <row r="240" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A240" s="4"/>
       <c r="B240" s="19"/>
       <c r="C240" s="4"/>
@@ -11104,7 +11115,7 @@
       <c r="AD240" s="4"/>
       <c r="AE240" s="4"/>
     </row>
-    <row r="241" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A241" s="4"/>
       <c r="B241" s="19"/>
       <c r="C241" s="4"/>
@@ -11137,7 +11148,7 @@
       <c r="AD241" s="4"/>
       <c r="AE241" s="4"/>
     </row>
-    <row r="242" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A242" s="4"/>
       <c r="B242" s="19"/>
       <c r="C242" s="4"/>
@@ -11170,7 +11181,7 @@
       <c r="AD242" s="4"/>
       <c r="AE242" s="4"/>
     </row>
-    <row r="243" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A243" s="4"/>
       <c r="B243" s="19"/>
       <c r="C243" s="4"/>
@@ -11203,7 +11214,7 @@
       <c r="AD243" s="4"/>
       <c r="AE243" s="4"/>
     </row>
-    <row r="244" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A244" s="4"/>
       <c r="B244" s="19"/>
       <c r="C244" s="4"/>
@@ -11236,7 +11247,7 @@
       <c r="AD244" s="4"/>
       <c r="AE244" s="4"/>
     </row>
-    <row r="245" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A245" s="4"/>
       <c r="B245" s="19"/>
       <c r="C245" s="4"/>
@@ -11269,7 +11280,7 @@
       <c r="AD245" s="4"/>
       <c r="AE245" s="4"/>
     </row>
-    <row r="246" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A246" s="4"/>
       <c r="B246" s="19"/>
       <c r="C246" s="4"/>
@@ -11302,7 +11313,7 @@
       <c r="AD246" s="4"/>
       <c r="AE246" s="4"/>
     </row>
-    <row r="247" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A247" s="4"/>
       <c r="B247" s="19"/>
       <c r="C247" s="4"/>
@@ -11335,7 +11346,7 @@
       <c r="AD247" s="4"/>
       <c r="AE247" s="4"/>
     </row>
-    <row r="248" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A248" s="4"/>
       <c r="B248" s="19"/>
       <c r="C248" s="4"/>
@@ -11368,7 +11379,7 @@
       <c r="AD248" s="4"/>
       <c r="AE248" s="4"/>
     </row>
-    <row r="249" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A249" s="4"/>
       <c r="B249" s="19"/>
       <c r="C249" s="4"/>
@@ -11401,7 +11412,7 @@
       <c r="AD249" s="4"/>
       <c r="AE249" s="4"/>
     </row>
-    <row r="250" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A250" s="4"/>
       <c r="B250" s="19"/>
       <c r="C250" s="4"/>
@@ -11434,7 +11445,7 @@
       <c r="AD250" s="4"/>
       <c r="AE250" s="4"/>
     </row>
-    <row r="251" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A251" s="4"/>
       <c r="B251" s="19"/>
       <c r="C251" s="4"/>
@@ -11467,7 +11478,7 @@
       <c r="AD251" s="4"/>
       <c r="AE251" s="4"/>
     </row>
-    <row r="252" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A252" s="4"/>
       <c r="B252" s="5"/>
       <c r="C252" s="4"/>
@@ -11500,7 +11511,7 @@
       <c r="AD252" s="4"/>
       <c r="AE252" s="4"/>
     </row>
-    <row r="253" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A253" s="4"/>
       <c r="B253" s="5"/>
       <c r="C253" s="4"/>
@@ -11533,7 +11544,7 @@
       <c r="AD253" s="4"/>
       <c r="AE253" s="4"/>
     </row>
-    <row r="254" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A254" s="4"/>
       <c r="B254" s="5"/>
       <c r="C254" s="4"/>
@@ -11566,7 +11577,7 @@
       <c r="AD254" s="4"/>
       <c r="AE254" s="4"/>
     </row>
-    <row r="255" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A255" s="4"/>
       <c r="B255" s="5"/>
       <c r="C255" s="4"/>
@@ -11599,7 +11610,7 @@
       <c r="AD255" s="4"/>
       <c r="AE255" s="4"/>
     </row>
-    <row r="256" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A256" s="4"/>
       <c r="B256" s="5"/>
       <c r="C256" s="4"/>
@@ -11632,7 +11643,7 @@
       <c r="AD256" s="4"/>
       <c r="AE256" s="4"/>
     </row>
-    <row r="257" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A257" s="4"/>
       <c r="B257" s="5"/>
       <c r="C257" s="4"/>
@@ -11665,7 +11676,7 @@
       <c r="AD257" s="4"/>
       <c r="AE257" s="4"/>
     </row>
-    <row r="258" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A258" s="4"/>
       <c r="B258" s="5"/>
       <c r="C258" s="4"/>
@@ -11698,7 +11709,7 @@
       <c r="AD258" s="4"/>
       <c r="AE258" s="4"/>
     </row>
-    <row r="259" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A259" s="4"/>
       <c r="B259" s="5"/>
       <c r="C259" s="4" t="s">
@@ -11735,7 +11746,7 @@
       <c r="AD259" s="4"/>
       <c r="AE259" s="4"/>
     </row>
-    <row r="260" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A260" s="4"/>
       <c r="B260" s="5"/>
       <c r="C260" s="4" t="s">
@@ -11770,7 +11781,7 @@
       <c r="AD260" s="4"/>
       <c r="AE260" s="4"/>
     </row>
-    <row r="261" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A261" s="4"/>
       <c r="B261" s="5"/>
       <c r="C261" s="4"/>
@@ -11803,7 +11814,7 @@
       <c r="AD261" s="4"/>
       <c r="AE261" s="4"/>
     </row>
-    <row r="262" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A262" s="4"/>
       <c r="B262" s="5"/>
       <c r="C262" s="4"/>
@@ -11839,7 +11850,7 @@
       <c r="AD262" s="4"/>
       <c r="AE262" s="4"/>
     </row>
-    <row r="263" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A263" s="4"/>
       <c r="B263" s="5"/>
       <c r="C263" s="4"/>
@@ -11872,7 +11883,7 @@
       <c r="AD263" s="4"/>
       <c r="AE263" s="4"/>
     </row>
-    <row r="264" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A264" s="4"/>
       <c r="B264" s="5"/>
       <c r="C264" s="4"/>
@@ -11905,7 +11916,7 @@
       <c r="AD264" s="4"/>
       <c r="AE264" s="4"/>
     </row>
-    <row r="265" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A265" s="4"/>
       <c r="B265" s="5"/>
       <c r="C265" s="4"/>
@@ -11938,7 +11949,7 @@
       <c r="AD265" s="4"/>
       <c r="AE265" s="4"/>
     </row>
-    <row r="266" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A266" s="4"/>
       <c r="B266" s="5"/>
       <c r="C266" s="4"/>
@@ -11971,7 +11982,7 @@
       <c r="AD266" s="4"/>
       <c r="AE266" s="4"/>
     </row>
-    <row r="267" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A267" s="4"/>
       <c r="B267" s="5"/>
       <c r="C267" s="4"/>
@@ -12004,7 +12015,7 @@
       <c r="AD267" s="4"/>
       <c r="AE267" s="4"/>
     </row>
-    <row r="268" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A268" s="4"/>
       <c r="B268" s="5"/>
       <c r="C268" s="4"/>
@@ -12037,7 +12048,7 @@
       <c r="AD268" s="4"/>
       <c r="AE268" s="4"/>
     </row>
-    <row r="269" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A269" s="4"/>
       <c r="B269" s="5"/>
       <c r="C269" s="4"/>
@@ -12070,7 +12081,7 @@
       <c r="AD269" s="4"/>
       <c r="AE269" s="4"/>
     </row>
-    <row r="270" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A270" s="4"/>
       <c r="B270" s="5"/>
       <c r="C270" s="4"/>
@@ -12103,7 +12114,7 @@
       <c r="AD270" s="4"/>
       <c r="AE270" s="4"/>
     </row>
-    <row r="271" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D271" s="6"/>
       <c r="E271" s="7"/>
       <c r="F271" s="5"/>
@@ -12133,7 +12144,7 @@
       <c r="AD271" s="4"/>
       <c r="AE271" s="4"/>
     </row>
-    <row r="272" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D272" s="6"/>
       <c r="E272" s="7"/>
       <c r="F272" s="5"/>
@@ -12163,7 +12174,7 @@
       <c r="AD272" s="4"/>
       <c r="AE272" s="4"/>
     </row>
-    <row r="273" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D273" s="6"/>
       <c r="E273" s="7"/>
       <c r="F273" s="5"/>
@@ -12193,7 +12204,7 @@
       <c r="AD273" s="4"/>
       <c r="AE273" s="4"/>
     </row>
-    <row r="274" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D274" s="6"/>
       <c r="E274" s="7"/>
       <c r="F274" s="5"/>
@@ -12223,7 +12234,7 @@
       <c r="AD274" s="4"/>
       <c r="AE274" s="4"/>
     </row>
-    <row r="275" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D275" s="6"/>
       <c r="E275" s="7"/>
       <c r="F275" s="5"/>
@@ -12253,7 +12264,7 @@
       <c r="AD275" s="4"/>
       <c r="AE275" s="4"/>
     </row>
-    <row r="276" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D276" s="6"/>
       <c r="E276" s="7"/>
       <c r="F276" s="5"/>
@@ -12283,7 +12294,7 @@
       <c r="AD276" s="4"/>
       <c r="AE276" s="4"/>
     </row>
-    <row r="277" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D277" s="6"/>
       <c r="E277" s="7"/>
       <c r="F277" s="5"/>
@@ -12313,7 +12324,7 @@
       <c r="AD277" s="4"/>
       <c r="AE277" s="4"/>
     </row>
-    <row r="278" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D278" s="6"/>
       <c r="E278" s="7"/>
       <c r="F278" s="5"/>
@@ -12343,7 +12354,7 @@
       <c r="AD278" s="4"/>
       <c r="AE278" s="4"/>
     </row>
-    <row r="279" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D279" s="6"/>
       <c r="E279" s="7"/>
       <c r="F279" s="5"/>
@@ -12373,7 +12384,7 @@
       <c r="AD279" s="4"/>
       <c r="AE279" s="4"/>
     </row>
-    <row r="280" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D280" s="6"/>
       <c r="E280" s="7"/>
       <c r="F280" s="5"/>
@@ -12403,7 +12414,7 @@
       <c r="AD280" s="4"/>
       <c r="AE280" s="4"/>
     </row>
-    <row r="281" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D281" s="6"/>
       <c r="E281" s="7"/>
       <c r="F281" s="5"/>
@@ -12433,7 +12444,7 @@
       <c r="AD281" s="4"/>
       <c r="AE281" s="4"/>
     </row>
-    <row r="282" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D282" s="6"/>
       <c r="E282" s="7"/>
       <c r="F282" s="5"/>
@@ -12463,7 +12474,7 @@
       <c r="AD282" s="4"/>
       <c r="AE282" s="4"/>
     </row>
-    <row r="283" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D283" s="6"/>
       <c r="E283" s="7"/>
       <c r="F283" s="5"/>
@@ -12493,7 +12504,7 @@
       <c r="AD283" s="4"/>
       <c r="AE283" s="4"/>
     </row>
-    <row r="284" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D284" s="6"/>
       <c r="E284" s="7"/>
       <c r="F284" s="5"/>
@@ -12523,7 +12534,7 @@
       <c r="AD284" s="4"/>
       <c r="AE284" s="4"/>
     </row>
-    <row r="285" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D285" s="6"/>
       <c r="E285" s="7"/>
       <c r="F285" s="5"/>
@@ -12553,7 +12564,7 @@
       <c r="AD285" s="4"/>
       <c r="AE285" s="4"/>
     </row>
-    <row r="286" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D286" s="6"/>
       <c r="E286" s="7"/>
       <c r="F286" s="5"/>
@@ -12583,7 +12594,7 @@
       <c r="AD286" s="4"/>
       <c r="AE286" s="4"/>
     </row>
-    <row r="287" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D287" s="6"/>
       <c r="E287" s="7"/>
       <c r="F287" s="5"/>
@@ -12613,7 +12624,7 @@
       <c r="AD287" s="4"/>
       <c r="AE287" s="4"/>
     </row>
-    <row r="288" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D288" s="6"/>
       <c r="E288" s="7"/>
       <c r="F288" s="5"/>
@@ -12643,7 +12654,7 @@
       <c r="AD288" s="4"/>
       <c r="AE288" s="4"/>
     </row>
-    <row r="289" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D289" s="6"/>
       <c r="E289" s="7"/>
       <c r="F289" s="5"/>
@@ -12673,7 +12684,7 @@
       <c r="AD289" s="4"/>
       <c r="AE289" s="4"/>
     </row>
-    <row r="290" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D290" s="6"/>
       <c r="E290" s="7"/>
       <c r="F290" s="5"/>
@@ -12703,7 +12714,7 @@
       <c r="AD290" s="4"/>
       <c r="AE290" s="4"/>
     </row>
-    <row r="291" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D291" s="6"/>
       <c r="E291" s="7"/>
       <c r="F291" s="5"/>
@@ -12733,7 +12744,7 @@
       <c r="AD291" s="4"/>
       <c r="AE291" s="4"/>
     </row>
-    <row r="292" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D292" s="6"/>
       <c r="E292" s="7"/>
       <c r="F292" s="5"/>
@@ -12763,7 +12774,7 @@
       <c r="AD292" s="4"/>
       <c r="AE292" s="4"/>
     </row>
-    <row r="293" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D293" s="6"/>
       <c r="E293" s="7"/>
       <c r="F293" s="5"/>
@@ -12793,7 +12804,7 @@
       <c r="AD293" s="4"/>
       <c r="AE293" s="4"/>
     </row>
-    <row r="294" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="4:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D294" s="6"/>
       <c r="E294" s="7"/>
       <c r="F294" s="5"/>
@@ -12825,11 +12836,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B12:K12"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="I30:J30"/>
     <mergeCell ref="O200:P200"/>
     <mergeCell ref="Q200:R200"/>
     <mergeCell ref="S200:T200"/>
@@ -12839,6 +12845,11 @@
     <mergeCell ref="C79:K79"/>
     <mergeCell ref="C82:K82"/>
     <mergeCell ref="B184:K184"/>
+    <mergeCell ref="B12:K12"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="I30:J30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(settings): upgrade typing_delay_ms to SafeSpinBox, add boundary keyword validation
- Change typing_delay_ms kind from 'text' to 'spinbox' in OIC automation
  defaults rows — prevents 'Yes'/'No' text accidentally entering a numeric field
- Add 'spinbox' widget handling in _load_data: creates SafeSpinBox(0-999)
  with ' ms' suffix and NoButtons (mouse-wheel safe), loads saved value
- Add QSpinBox isinstance path in _save_all: reads widget.value() as int,
  saves as numeric string — no text parsing or manual validation needed
- Remove redundant typing_delay_ms text validation (spinbox enforces constraint)
- Add table_boundary_keyword validation: blocks empty value and Yes/No/True/False
  accidental inputs that caused the boundary-stop bug (root cause of Claim number
  leak into assessment output)
- Full end-to-end audit passed: all 16 OIC defaults Load -> Save -> Use verified
</commit_message>
<xml_diff>
--- a/OIC DOCS/dummy.xlsx
+++ b/OIC DOCS/dummy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jadav\Coding\Automation\UIIC\uiic_automation\OIC DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E86E18-178E-485C-9405-7C1D21E7DE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74C5E2C4-DE6A-47E9-90AE-955D89370F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1634,27 +1634,60 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1663,39 +1696,6 @@
     </xf>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2385,18 +2385,18 @@
     </row>
     <row r="12" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
-      <c r="B12" s="151" t="s">
+      <c r="B12" s="168" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="152"/>
-      <c r="D12" s="153"/>
-      <c r="E12" s="154"/>
-      <c r="F12" s="155"/>
-      <c r="G12" s="155"/>
-      <c r="H12" s="154"/>
-      <c r="I12" s="154"/>
-      <c r="J12" s="154"/>
-      <c r="K12" s="155"/>
+      <c r="C12" s="167"/>
+      <c r="D12" s="163"/>
+      <c r="E12" s="164"/>
+      <c r="F12" s="165"/>
+      <c r="G12" s="165"/>
+      <c r="H12" s="164"/>
+      <c r="I12" s="164"/>
+      <c r="J12" s="164"/>
+      <c r="K12" s="165"/>
       <c r="L12" s="4"/>
       <c r="M12" s="5"/>
       <c r="N12" s="7"/>
@@ -3051,14 +3051,14 @@
       <c r="D29" s="28"/>
       <c r="E29" s="29"/>
       <c r="F29" s="30"/>
-      <c r="G29" s="156" t="s">
+      <c r="G29" s="159" t="s">
         <v>41</v>
       </c>
-      <c r="H29" s="157"/>
-      <c r="I29" s="158" t="s">
+      <c r="H29" s="152"/>
+      <c r="I29" s="169" t="s">
         <v>42</v>
       </c>
-      <c r="J29" s="157"/>
+      <c r="J29" s="152"/>
       <c r="K29" s="31" t="s">
         <v>43</v>
       </c>
@@ -3096,15 +3096,15 @@
       <c r="F30" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="G30" s="159" t="s">
+      <c r="G30" s="170" t="s">
         <v>45</v>
       </c>
-      <c r="H30" s="160"/>
-      <c r="I30" s="158" t="str">
+      <c r="H30" s="171"/>
+      <c r="I30" s="169" t="str">
         <f>G30</f>
         <v>MEXC19606KT080595</v>
       </c>
-      <c r="J30" s="157"/>
+      <c r="J30" s="152"/>
       <c r="K30" s="31" t="str">
         <f>G30</f>
         <v>MEXC19606KT080595</v>
@@ -3143,15 +3143,15 @@
       <c r="F31" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="G31" s="156" t="s">
+      <c r="G31" s="159" t="s">
         <v>48</v>
       </c>
-      <c r="H31" s="157"/>
-      <c r="I31" s="168" t="str">
+      <c r="H31" s="152"/>
+      <c r="I31" s="160" t="str">
         <f>G31</f>
         <v>CBZL12533</v>
       </c>
-      <c r="J31" s="169"/>
+      <c r="J31" s="161"/>
       <c r="K31" s="37" t="str">
         <f>G31</f>
         <v>CBZL12533</v>
@@ -5099,17 +5099,17 @@
     <row r="79" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4"/>
       <c r="B79" s="19"/>
-      <c r="C79" s="170" t="s">
+      <c r="C79" s="162" t="s">
         <v>16</v>
       </c>
-      <c r="D79" s="153"/>
-      <c r="E79" s="154"/>
-      <c r="F79" s="155"/>
-      <c r="G79" s="155"/>
-      <c r="H79" s="154"/>
-      <c r="I79" s="154"/>
-      <c r="J79" s="154"/>
-      <c r="K79" s="155"/>
+      <c r="D79" s="163"/>
+      <c r="E79" s="164"/>
+      <c r="F79" s="165"/>
+      <c r="G79" s="165"/>
+      <c r="H79" s="164"/>
+      <c r="I79" s="164"/>
+      <c r="J79" s="164"/>
+      <c r="K79" s="165"/>
       <c r="L79" s="4"/>
       <c r="M79" s="5"/>
       <c r="N79" s="7"/>
@@ -5212,17 +5212,17 @@
     <row r="82" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4"/>
       <c r="B82" s="19"/>
-      <c r="C82" s="170" t="s">
+      <c r="C82" s="162" t="s">
         <v>147</v>
       </c>
-      <c r="D82" s="153"/>
-      <c r="E82" s="154"/>
-      <c r="F82" s="155"/>
-      <c r="G82" s="155"/>
-      <c r="H82" s="154"/>
-      <c r="I82" s="154"/>
-      <c r="J82" s="154"/>
-      <c r="K82" s="155"/>
+      <c r="D82" s="163"/>
+      <c r="E82" s="164"/>
+      <c r="F82" s="165"/>
+      <c r="G82" s="165"/>
+      <c r="H82" s="164"/>
+      <c r="I82" s="164"/>
+      <c r="J82" s="164"/>
+      <c r="K82" s="165"/>
       <c r="L82" s="4"/>
       <c r="M82" s="5"/>
       <c r="N82" s="7"/>
@@ -6066,13 +6066,9 @@
       <c r="F104" s="72">
         <v>8861</v>
       </c>
-      <c r="G104" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H104" s="72">
+      <c r="I104" s="3">
         <v>5</v>
       </c>
-      <c r="I104" s="72"/>
       <c r="J104" s="7"/>
       <c r="K104" s="5"/>
       <c r="L104" s="4"/>
@@ -6109,13 +6105,6 @@
       <c r="F105" s="72">
         <v>9110</v>
       </c>
-      <c r="G105" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H105" s="72">
-        <v>5</v>
-      </c>
-      <c r="I105" s="72"/>
       <c r="J105" s="7"/>
       <c r="K105" s="5"/>
       <c r="L105" s="4"/>
@@ -6152,13 +6141,6 @@
       <c r="F106" s="72">
         <v>3030</v>
       </c>
-      <c r="G106" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H106" s="72">
-        <v>4</v>
-      </c>
-      <c r="I106" s="72"/>
       <c r="J106" s="7"/>
       <c r="K106" s="5"/>
       <c r="L106" s="4"/>
@@ -6195,20 +6177,17 @@
       <c r="F107" s="72">
         <v>1560</v>
       </c>
-      <c r="G107" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H107" s="72"/>
-      <c r="I107" s="72">
-        <v>5</v>
-      </c>
       <c r="J107" s="7"/>
       <c r="K107" s="5"/>
       <c r="L107" s="4"/>
       <c r="M107" s="5"/>
-      <c r="N107" s="7"/>
-      <c r="O107" s="5"/>
-      <c r="P107" s="7"/>
+      <c r="N107" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O107" s="72">
+        <v>5</v>
+      </c>
+      <c r="P107" s="72"/>
       <c r="Q107" s="5"/>
       <c r="R107" s="7"/>
       <c r="S107" s="4"/>
@@ -6238,20 +6217,17 @@
       <c r="F108" s="72">
         <v>8570</v>
       </c>
-      <c r="G108" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H108" s="72">
-        <v>4</v>
-      </c>
-      <c r="I108" s="72"/>
       <c r="J108" s="7"/>
       <c r="K108" s="5"/>
       <c r="L108" s="4"/>
       <c r="M108" s="5"/>
-      <c r="N108" s="7"/>
-      <c r="O108" s="5"/>
-      <c r="P108" s="7"/>
+      <c r="N108" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O108" s="72">
+        <v>5</v>
+      </c>
+      <c r="P108" s="72"/>
       <c r="Q108" s="5"/>
       <c r="R108" s="7"/>
       <c r="S108" s="4"/>
@@ -6281,20 +6257,17 @@
       <c r="F109" s="72">
         <v>9110</v>
       </c>
-      <c r="G109" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H109" s="72">
-        <v>4</v>
-      </c>
-      <c r="I109" s="72"/>
       <c r="J109" s="7"/>
       <c r="K109" s="5"/>
       <c r="L109" s="4"/>
       <c r="M109" s="5"/>
-      <c r="N109" s="7"/>
-      <c r="O109" s="5"/>
-      <c r="P109" s="7"/>
+      <c r="N109" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O109" s="72">
+        <v>4</v>
+      </c>
+      <c r="P109" s="72"/>
       <c r="Q109" s="5"/>
       <c r="R109" s="7"/>
       <c r="S109" s="4"/>
@@ -6324,20 +6297,17 @@
       <c r="F110" s="72">
         <v>8861</v>
       </c>
-      <c r="G110" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H110" s="72"/>
-      <c r="I110" s="72">
-        <v>5</v>
-      </c>
       <c r="J110" s="7"/>
       <c r="K110" s="5"/>
       <c r="L110" s="4"/>
       <c r="M110" s="5"/>
-      <c r="N110" s="7"/>
-      <c r="O110" s="5"/>
-      <c r="P110" s="7"/>
+      <c r="N110" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O110" s="72"/>
+      <c r="P110" s="72">
+        <v>5</v>
+      </c>
       <c r="Q110" s="5"/>
       <c r="R110" s="7"/>
       <c r="S110" s="4"/>
@@ -6367,20 +6337,17 @@
       <c r="F111" s="72">
         <v>2270</v>
       </c>
-      <c r="G111" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H111" s="72"/>
-      <c r="I111" s="72">
-        <v>4</v>
-      </c>
       <c r="J111" s="7"/>
       <c r="K111" s="5"/>
       <c r="L111" s="4"/>
       <c r="M111" s="5"/>
-      <c r="N111" s="7"/>
-      <c r="O111" s="5"/>
-      <c r="P111" s="7"/>
+      <c r="N111" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O111" s="72">
+        <v>4</v>
+      </c>
+      <c r="P111" s="72"/>
       <c r="Q111" s="5"/>
       <c r="R111" s="7"/>
       <c r="S111" s="4"/>
@@ -6410,20 +6377,17 @@
       <c r="F112" s="72">
         <v>2270</v>
       </c>
-      <c r="G112" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H112" s="72">
-        <v>5</v>
-      </c>
-      <c r="I112" s="72"/>
       <c r="J112" s="7"/>
       <c r="K112" s="5"/>
       <c r="L112" s="4"/>
       <c r="M112" s="5"/>
-      <c r="N112" s="7"/>
-      <c r="O112" s="5"/>
-      <c r="P112" s="7"/>
+      <c r="N112" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O112" s="72">
+        <v>4</v>
+      </c>
+      <c r="P112" s="72"/>
       <c r="Q112" s="5"/>
       <c r="R112" s="7"/>
       <c r="S112" s="4"/>
@@ -6453,20 +6417,17 @@
       <c r="F113" s="72">
         <v>302</v>
       </c>
-      <c r="G113" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H113" s="72">
-        <v>4</v>
-      </c>
-      <c r="I113" s="72"/>
       <c r="J113" s="7"/>
       <c r="K113" s="5"/>
       <c r="L113" s="4"/>
       <c r="M113" s="5"/>
-      <c r="N113" s="7"/>
-      <c r="O113" s="5"/>
-      <c r="P113" s="7"/>
+      <c r="N113" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O113" s="72"/>
+      <c r="P113" s="72">
+        <v>5</v>
+      </c>
       <c r="Q113" s="5"/>
       <c r="R113" s="7"/>
       <c r="S113" s="4"/>
@@ -6496,20 +6457,17 @@
       <c r="F114" s="72">
         <v>3560</v>
       </c>
-      <c r="G114" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H114" s="72"/>
-      <c r="I114" s="72">
-        <v>5</v>
-      </c>
       <c r="J114" s="7"/>
       <c r="K114" s="5"/>
       <c r="L114" s="4"/>
       <c r="M114" s="5"/>
-      <c r="N114" s="7"/>
-      <c r="O114" s="5"/>
-      <c r="P114" s="7"/>
+      <c r="N114" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O114" s="72"/>
+      <c r="P114" s="72">
+        <v>4</v>
+      </c>
       <c r="Q114" s="5"/>
       <c r="R114" s="7"/>
       <c r="S114" s="4"/>
@@ -6539,20 +6497,17 @@
       <c r="F115" s="72">
         <v>70000</v>
       </c>
-      <c r="G115" s="75" t="s">
-        <v>175</v>
-      </c>
-      <c r="H115" s="72">
-        <v>4</v>
-      </c>
-      <c r="I115" s="72"/>
       <c r="J115" s="7"/>
       <c r="K115" s="5"/>
       <c r="L115" s="4"/>
       <c r="M115" s="5"/>
-      <c r="N115" s="7"/>
-      <c r="O115" s="5"/>
-      <c r="P115" s="7"/>
+      <c r="N115" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O115" s="72">
+        <v>5</v>
+      </c>
+      <c r="P115" s="72"/>
       <c r="Q115" s="5"/>
       <c r="R115" s="7"/>
       <c r="S115" s="4"/>
@@ -6582,11 +6537,6 @@
       <c r="F116" s="72">
         <v>100</v>
       </c>
-      <c r="G116" s="72"/>
-      <c r="H116" s="72">
-        <v>4</v>
-      </c>
-      <c r="I116" s="72"/>
       <c r="J116" s="76">
         <v>1771.18</v>
       </c>
@@ -6595,9 +6545,13 @@
       </c>
       <c r="L116" s="4"/>
       <c r="M116" s="5"/>
-      <c r="N116" s="7"/>
-      <c r="O116" s="5"/>
-      <c r="P116" s="7"/>
+      <c r="N116" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O116" s="72">
+        <v>4</v>
+      </c>
+      <c r="P116" s="72"/>
       <c r="Q116" s="5"/>
       <c r="R116" s="7"/>
       <c r="S116" s="4"/>
@@ -6627,11 +6581,6 @@
       <c r="F117" s="72">
         <v>12</v>
       </c>
-      <c r="G117" s="72"/>
-      <c r="H117" s="72"/>
-      <c r="I117" s="72">
-        <v>4</v>
-      </c>
       <c r="J117" s="69">
         <v>20000</v>
       </c>
@@ -6640,9 +6589,13 @@
       </c>
       <c r="L117" s="4"/>
       <c r="M117" s="5"/>
-      <c r="N117" s="7"/>
-      <c r="O117" s="5"/>
-      <c r="P117" s="7"/>
+      <c r="N117" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O117" s="72"/>
+      <c r="P117" s="72">
+        <v>5</v>
+      </c>
       <c r="Q117" s="5"/>
       <c r="R117" s="7"/>
       <c r="S117" s="4"/>
@@ -6672,18 +6625,17 @@
       <c r="F118" s="72">
         <v>150</v>
       </c>
-      <c r="G118" s="72"/>
-      <c r="H118" s="72">
-        <v>500</v>
-      </c>
-      <c r="I118" s="72"/>
       <c r="J118" s="7"/>
       <c r="K118" s="5"/>
       <c r="L118" s="4"/>
       <c r="M118" s="5"/>
-      <c r="N118" s="7"/>
-      <c r="O118" s="5"/>
-      <c r="P118" s="7"/>
+      <c r="N118" s="75" t="s">
+        <v>175</v>
+      </c>
+      <c r="O118" s="72">
+        <v>4</v>
+      </c>
+      <c r="P118" s="72"/>
       <c r="Q118" s="5"/>
       <c r="R118" s="7"/>
       <c r="S118" s="4"/>
@@ -6714,9 +6666,11 @@
       <c r="K119" s="5"/>
       <c r="L119" s="4"/>
       <c r="M119" s="5"/>
-      <c r="N119" s="7"/>
-      <c r="O119" s="5"/>
-      <c r="P119" s="7"/>
+      <c r="N119" s="72"/>
+      <c r="O119" s="72">
+        <v>4</v>
+      </c>
+      <c r="P119" s="72"/>
       <c r="Q119" s="5"/>
       <c r="R119" s="7"/>
       <c r="S119" s="4"/>
@@ -6747,9 +6701,11 @@
       <c r="K120" s="5"/>
       <c r="L120" s="4"/>
       <c r="M120" s="5"/>
-      <c r="N120" s="7"/>
-      <c r="O120" s="5"/>
-      <c r="P120" s="7"/>
+      <c r="N120" s="72"/>
+      <c r="O120" s="72"/>
+      <c r="P120" s="72">
+        <v>4</v>
+      </c>
       <c r="Q120" s="5"/>
       <c r="R120" s="7"/>
       <c r="S120" s="4"/>
@@ -6780,9 +6736,11 @@
       <c r="K121" s="5"/>
       <c r="L121" s="4"/>
       <c r="M121" s="5"/>
-      <c r="N121" s="7"/>
-      <c r="O121" s="5"/>
-      <c r="P121" s="7"/>
+      <c r="N121" s="72"/>
+      <c r="O121" s="72">
+        <v>500</v>
+      </c>
+      <c r="P121" s="72"/>
       <c r="Q121" s="5"/>
       <c r="R121" s="7"/>
       <c r="S121" s="4"/>
@@ -7281,11 +7239,11 @@
       </c>
       <c r="H136" s="84">
         <f>SUM(H101:H135)</f>
-        <v>1039</v>
+        <v>500</v>
       </c>
       <c r="I136" s="84">
         <f>SUM(I101:I135)</f>
-        <v>1023</v>
+        <v>1005</v>
       </c>
       <c r="J136" s="56">
         <f>SUM(J101:J135)</f>
@@ -7333,11 +7291,11 @@
       </c>
       <c r="H137" s="87">
         <f>B137*H136/100</f>
-        <v>187.02</v>
+        <v>90</v>
       </c>
       <c r="I137" s="87">
         <f>18*I136/100</f>
-        <v>184.14</v>
+        <v>180.9</v>
       </c>
       <c r="J137" s="56"/>
       <c r="K137" s="5"/>
@@ -7380,11 +7338,11 @@
       </c>
       <c r="H138" s="83">
         <f>SUM(H136:H137)</f>
-        <v>1226.02</v>
+        <v>590</v>
       </c>
       <c r="I138" s="84">
         <f>SUM(I136:I137)</f>
-        <v>1207.1399999999999</v>
+        <v>1185.9000000000001</v>
       </c>
       <c r="J138" s="56"/>
       <c r="K138" s="5"/>
@@ -7462,7 +7420,7 @@
       </c>
       <c r="H140" s="90">
         <f>H138/2</f>
-        <v>613.01</v>
+        <v>295</v>
       </c>
       <c r="I140" s="84">
         <v>0</v>
@@ -7508,11 +7466,11 @@
       </c>
       <c r="H141" s="92">
         <f>H138-H140</f>
-        <v>613.01</v>
+        <v>295</v>
       </c>
       <c r="I141" s="93">
         <f>I138-I140</f>
-        <v>1207.1399999999999</v>
+        <v>1185.9000000000001</v>
       </c>
       <c r="J141" s="56"/>
       <c r="K141" s="5"/>
@@ -7551,7 +7509,7 @@
       </c>
       <c r="G142" s="96">
         <f>G141+H141+I141+J141</f>
-        <v>4419.8197999999993</v>
+        <v>4080.5698000000002</v>
       </c>
       <c r="H142" s="97"/>
       <c r="I142" s="91"/>
@@ -7622,7 +7580,7 @@
       <c r="F144" s="5"/>
       <c r="G144" s="20">
         <f>G140+H140+J140+I140</f>
-        <v>613.01</v>
+        <v>295</v>
       </c>
       <c r="H144" s="7"/>
       <c r="I144" s="7"/>
@@ -8762,7 +8720,7 @@
       </c>
       <c r="G175" s="112">
         <f>G142</f>
-        <v>4419.8197999999993</v>
+        <v>4080.5698000000002</v>
       </c>
       <c r="H175" s="7"/>
       <c r="I175" s="7"/>
@@ -8844,7 +8802,7 @@
       </c>
       <c r="G177" s="72">
         <f>G175+G176</f>
-        <v>4437.5197999999991</v>
+        <v>4098.2698</v>
       </c>
       <c r="H177" s="7"/>
       <c r="I177" s="7"/>
@@ -8923,7 +8881,7 @@
       </c>
       <c r="G179" s="121">
         <f>G177-G178</f>
-        <v>3937.5197999999991</v>
+        <v>3598.2698</v>
       </c>
       <c r="H179" s="7"/>
       <c r="I179" s="7"/>
@@ -9031,7 +8989,7 @@
       <c r="F182" s="53"/>
       <c r="G182" s="68">
         <f>G179-G181</f>
-        <v>3937.5197999999991</v>
+        <v>3598.2698</v>
       </c>
       <c r="H182" s="7"/>
       <c r="I182" s="56"/>
@@ -9093,18 +9051,18 @@
     </row>
     <row r="184" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="4"/>
-      <c r="B184" s="171" t="s">
+      <c r="B184" s="166" t="s">
         <v>219</v>
       </c>
-      <c r="C184" s="152"/>
-      <c r="D184" s="153"/>
-      <c r="E184" s="154"/>
-      <c r="F184" s="155"/>
-      <c r="G184" s="155"/>
-      <c r="H184" s="154"/>
-      <c r="I184" s="154"/>
-      <c r="J184" s="154"/>
-      <c r="K184" s="155"/>
+      <c r="C184" s="167"/>
+      <c r="D184" s="163"/>
+      <c r="E184" s="164"/>
+      <c r="F184" s="165"/>
+      <c r="G184" s="165"/>
+      <c r="H184" s="164"/>
+      <c r="I184" s="164"/>
+      <c r="J184" s="164"/>
+      <c r="K184" s="165"/>
       <c r="L184" s="4"/>
       <c r="M184" s="5"/>
       <c r="N184" s="7"/>
@@ -9678,22 +9636,22 @@
       <c r="N200" s="130" t="s">
         <v>229</v>
       </c>
-      <c r="O200" s="161" t="s">
+      <c r="O200" s="151" t="s">
         <v>230</v>
       </c>
-      <c r="P200" s="157"/>
-      <c r="Q200" s="161" t="s">
+      <c r="P200" s="152"/>
+      <c r="Q200" s="151" t="s">
         <v>231</v>
       </c>
-      <c r="R200" s="157"/>
-      <c r="S200" s="162" t="s">
+      <c r="R200" s="152"/>
+      <c r="S200" s="153" t="s">
         <v>232</v>
       </c>
-      <c r="T200" s="163"/>
-      <c r="U200" s="164" t="s">
+      <c r="T200" s="154"/>
+      <c r="U200" s="155" t="s">
         <v>233</v>
       </c>
-      <c r="V200" s="165"/>
+      <c r="V200" s="156"/>
       <c r="W200" s="4"/>
       <c r="X200" s="4"/>
       <c r="Y200" s="4"/>
@@ -9737,8 +9695,8 @@
       <c r="T201" s="136" t="s">
         <v>235</v>
       </c>
-      <c r="U201" s="166"/>
-      <c r="V201" s="167"/>
+      <c r="U201" s="157"/>
+      <c r="V201" s="158"/>
       <c r="W201" s="4"/>
       <c r="X201" s="4"/>
       <c r="Y201" s="4"/>
@@ -9769,27 +9727,27 @@
       <c r="M202" s="137"/>
       <c r="N202" s="43">
         <f>G136+H136</f>
-        <v>3242.11</v>
+        <v>2703.11</v>
       </c>
       <c r="O202" s="137">
         <v>14</v>
       </c>
       <c r="P202" s="138">
         <f>14*N202/100</f>
-        <v>453.8954</v>
+        <v>378.43540000000002</v>
       </c>
       <c r="Q202" s="139">
         <v>14</v>
       </c>
       <c r="R202" s="138">
         <f>P202</f>
-        <v>453.8954</v>
+        <v>378.43540000000002</v>
       </c>
       <c r="S202" s="70"/>
       <c r="T202" s="85"/>
       <c r="U202" s="56">
         <f>P202+R202</f>
-        <v>907.79079999999999</v>
+        <v>756.87080000000003</v>
       </c>
       <c r="V202" s="85"/>
       <c r="W202" s="4"/>
@@ -9818,27 +9776,27 @@
       <c r="M203" s="137"/>
       <c r="N203" s="43">
         <f>I136</f>
-        <v>1023</v>
+        <v>1005</v>
       </c>
       <c r="O203" s="137">
         <v>9</v>
       </c>
       <c r="P203" s="138">
         <f>9*N203/100</f>
-        <v>92.07</v>
+        <v>90.45</v>
       </c>
       <c r="Q203" s="139">
         <v>9</v>
       </c>
       <c r="R203" s="138">
         <f>P203</f>
-        <v>92.07</v>
+        <v>90.45</v>
       </c>
       <c r="S203" s="74"/>
       <c r="T203" s="85"/>
       <c r="U203" s="56">
         <f>P203+R203</f>
-        <v>184.14</v>
+        <v>180.9</v>
       </c>
       <c r="V203" s="85"/>
       <c r="W203" s="4"/>
@@ -9980,7 +9938,7 @@
       <c r="T206" s="101"/>
       <c r="U206" s="99">
         <f>SUM(U202:U205)</f>
-        <v>5013.4431999999997</v>
+        <v>4859.2831999999999</v>
       </c>
       <c r="V206" s="147"/>
       <c r="W206" s="4"/>
@@ -12836,6 +12794,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B12:K12"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="I30:J30"/>
     <mergeCell ref="O200:P200"/>
     <mergeCell ref="Q200:R200"/>
     <mergeCell ref="S200:T200"/>
@@ -12845,11 +12808,6 @@
     <mergeCell ref="C79:K79"/>
     <mergeCell ref="C82:K82"/>
     <mergeCell ref="B184:K184"/>
-    <mergeCell ref="B12:K12"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="I30:J30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>